<commit_message>
modified:   .gitignore modified:   data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx modified:   data/chapter2/FRED/subsets/species.xlsx deleted:    plots/995_species_5states_mapped_phylogeny.png deleted:    plots/DeltaLogRDvsStates.png deleted:    plots/DeltaLogSRLvsStates.png deleted:    plots/RD_SRL_dist.png deleted:    plots/emma_themeda_locations.jpeg deleted:    plots/emma_themeda_subset_soil_texture.jpeg deleted:    plots/emma_vin_themeda_locations.jpeg deleted:    plots/houwie_model_summary_100sims.png deleted:    plots/houwie_summary_rd_995sp_100sims.png deleted:    plots/houwie_summary_srl_995sp_100sims.png deleted:    plots/jay.png deleted:    plots/matmap6.png deleted:    plots/paired_independent_aces_all.png deleted:    plots/phosph.png deleted:    plots/power.png deleted:    plots/reciprocal.png deleted:    plots/roottraits.png deleted:    plots/themeda_site_props.png
</commit_message>
<xml_diff>
--- a/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
+++ b/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1613E9C1-AFA1-4AD8-8784-E6DED30E6CAB}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF889681-845B-4B0E-AD38-94737A5407DF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Information" sheetId="7" r:id="rId1"/>
@@ -4585,7 +4585,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -4603,41 +4603,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFC4D79B"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FFC4D79B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFC4D79B"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FFC4D79B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFC4D79B"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFC4D79B"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FFC4D79B"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -4652,7 +4617,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -4718,43 +4683,10 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4768,9 +4700,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4791,11 +4720,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4803,7 +4747,80 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFEBF1DE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FFC4D79B"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFC4D79B"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFC4D79B"/>
+        </left>
+        <top style="medium">
+          <color rgb="FFC4D79B"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFC4D79B"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border outline="0">
         <right style="thin">
@@ -4842,7 +4859,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I439" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I439" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A1:I439" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I439">
     <sortCondition ref="B1:B439"/>
@@ -4859,6 +4876,24 @@
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2922BC0C-E417-4658-AC0E-62ECDF39ADC6}" name="Table2" displayName="Table2" ref="A2:F89" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="8" tableBorderDxfId="9">
+  <autoFilter ref="A2:F89" xr:uid="{2922BC0C-E417-4658-AC0E-62ECDF39ADC6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F89">
+    <sortCondition ref="B2:B89"/>
+  </sortState>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{0BA76706-F6AC-4480-A1EA-EFC458A86717}" name="Order" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{5641DCB1-A433-40BD-9ED9-D33902929B8C}" name="Family" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{DAAE68C8-09E1-4B56-912D-11D87EB83220}" name="Habit" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{2BC3EF26-068C-475F-91C7-4E8D11F95517}" name="Ecology" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{C1FBDF6D-8E5A-4A09-BBA3-846E464D6CA5}" name="NM-AM" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{0B4BCA8E-55FF-4900-A159-74CFB7CBAE73}" name="NM" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -5165,12 +5200,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="36" customHeight="1">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="48" t="s">
         <v>1289</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="22" customHeight="1">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="47" t="s">
         <v>1238</v>
       </c>
     </row>
@@ -5332,7 +5367,7 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="62" t="s">
+      <c r="K1" s="50" t="s">
         <v>1246</v>
       </c>
     </row>
@@ -6304,7 +6339,7 @@
       <c r="F42" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H42" s="55"/>
+      <c r="H42" s="43"/>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
@@ -7372,56 +7407,56 @@
       </c>
     </row>
     <row r="90" spans="1:9">
-      <c r="A90" s="58" t="s">
+      <c r="A90" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="B90" s="58" t="s">
+      <c r="B90" s="46" t="s">
         <v>148</v>
       </c>
-      <c r="C90" s="58">
+      <c r="C90" s="46">
         <v>195</v>
       </c>
-      <c r="D90" s="58">
+      <c r="D90" s="46">
         <v>2</v>
       </c>
-      <c r="E90" s="58">
+      <c r="E90" s="46">
         <v>71</v>
       </c>
-      <c r="F90" s="58" t="s">
+      <c r="F90" s="46" t="s">
         <v>149</v>
       </c>
-      <c r="G90" s="58"/>
+      <c r="G90" s="46"/>
       <c r="H90" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="I90" s="58" t="s">
+      <c r="I90" s="46" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:9">
-      <c r="A91" s="58" t="s">
+      <c r="A91" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="B91" s="58" t="s">
+      <c r="B91" s="46" t="s">
         <v>148</v>
       </c>
-      <c r="C91" s="58">
+      <c r="C91" s="46">
         <v>195</v>
       </c>
-      <c r="D91" s="58">
+      <c r="D91" s="46">
         <v>2</v>
       </c>
-      <c r="E91" s="58">
+      <c r="E91" s="46">
         <v>20</v>
       </c>
-      <c r="F91" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="G91" s="58"/>
+      <c r="F91" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="G91" s="46"/>
       <c r="H91" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="I91" s="58" t="s">
+      <c r="I91" s="46" t="s">
         <v>1283</v>
       </c>
     </row>
@@ -7459,7 +7494,7 @@
       <c r="D93" s="5">
         <v>3</v>
       </c>
-      <c r="E93" s="56"/>
+      <c r="E93" s="44"/>
       <c r="F93" s="5" t="s">
         <v>12</v>
       </c>
@@ -8263,7 +8298,7 @@
       <c r="G127" s="8" t="s">
         <v>1225</v>
       </c>
-      <c r="H127" s="63" t="s">
+      <c r="H127" s="51" t="s">
         <v>1276</v>
       </c>
       <c r="I127" s="8" t="s">
@@ -15581,1621 +15616,1624 @@
   <dimension ref="A1:G90"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.9140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.9140625" customWidth="1"/>
+    <col min="5" max="5" width="11.08203125" customWidth="1"/>
+    <col min="6" max="6" width="8.9140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="82" customHeight="1" thickBot="1">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="52" t="s">
         <v>560</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
       <c r="G1" s="8" t="s">
         <v>1261</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" thickBot="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="37" t="s">
+      <c r="B2" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="58" t="s">
         <v>561</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="58" t="s">
         <v>562</v>
       </c>
-      <c r="E2" s="52" t="s">
+      <c r="E2" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="58" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" thickBot="1">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E3" s="36">
+        <v>2</v>
+      </c>
+      <c r="F3" s="55"/>
+    </row>
+    <row r="4" spans="1:7" ht="16" thickBot="1">
+      <c r="A4" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>590</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>591</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>592</v>
+      </c>
+      <c r="E4" s="55"/>
+      <c r="F4" s="36">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="16" thickBot="1">
+      <c r="A5" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E5" s="35">
+        <v>115</v>
+      </c>
+      <c r="F5" s="54"/>
+    </row>
+    <row r="6" spans="1:7" ht="16" thickBot="1">
+      <c r="A6" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>593</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>594</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>595</v>
+      </c>
+      <c r="E6" s="55"/>
+      <c r="F6" s="36">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" thickBot="1">
+      <c r="A7" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="E7" s="54"/>
+      <c r="F7" s="35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16" thickBot="1">
+      <c r="A8" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E8" s="36">
+        <v>56</v>
+      </c>
+      <c r="F8" s="55"/>
+    </row>
+    <row r="9" spans="1:7" ht="16" thickBot="1">
+      <c r="A9" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>571</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>572</v>
+      </c>
+      <c r="E9" s="35">
+        <v>1300</v>
+      </c>
+      <c r="F9" s="54"/>
+    </row>
+    <row r="10" spans="1:7" ht="16" thickBot="1">
+      <c r="A10" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="36" t="s">
+        <v>622</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>573</v>
+      </c>
+      <c r="E10" s="55"/>
+      <c r="F10" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16" thickBot="1">
+      <c r="A11" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="E11" s="54"/>
+      <c r="F11" s="35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="16" thickBot="1">
+      <c r="A12" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D12" s="35" t="s">
+        <v>617</v>
+      </c>
+      <c r="E12" s="54"/>
+      <c r="F12" s="35">
+        <v>3628</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="16" thickBot="1">
+      <c r="A13" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="E13" s="56">
+        <v>3475</v>
+      </c>
+      <c r="F13" s="54"/>
+    </row>
+    <row r="14" spans="1:7" ht="16" thickBot="1">
+      <c r="A14" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E14" s="36">
+        <v>1</v>
+      </c>
+      <c r="F14" s="55"/>
+    </row>
+    <row r="15" spans="1:7" ht="16" thickBot="1">
+      <c r="A15" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E15" s="54"/>
+      <c r="F15" s="35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="16" thickBot="1">
+      <c r="A16" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>623</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>573</v>
+      </c>
+      <c r="E16" s="36">
+        <v>75</v>
+      </c>
+      <c r="F16" s="55"/>
+    </row>
+    <row r="17" spans="1:6" ht="16" thickBot="1">
+      <c r="A17" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="36" t="s">
+        <v>587</v>
+      </c>
+      <c r="D17" s="36" t="s">
+        <v>618</v>
+      </c>
+      <c r="E17" s="55"/>
+      <c r="F17" s="36">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" thickBot="1">
+      <c r="A18" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>596</v>
+      </c>
+      <c r="E18" s="54"/>
+      <c r="F18" s="35">
+        <v>2625</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16" thickBot="1">
+      <c r="A19" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>599</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E19" s="54"/>
+      <c r="F19" s="35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16" thickBot="1">
+      <c r="A20" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D20" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E20" s="55"/>
+      <c r="F20" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16" thickBot="1">
+      <c r="A21" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>594</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>592</v>
+      </c>
+      <c r="E21" s="54"/>
+      <c r="F21" s="35">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16" thickBot="1">
+      <c r="A22" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>577</v>
+      </c>
+      <c r="E22" s="55"/>
+      <c r="F22" s="36">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="16" thickBot="1">
+      <c r="A23" s="36" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>626</v>
+      </c>
+      <c r="C23" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="D23" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E23" s="55"/>
+      <c r="F23" s="36">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="16" thickBot="1">
+      <c r="A24" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="35" t="s">
+        <v>181</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>594</v>
+      </c>
+      <c r="D24" s="35" t="s">
+        <v>611</v>
+      </c>
+      <c r="E24" s="35" t="s">
+        <v>612</v>
+      </c>
+      <c r="F24" s="35">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16" thickBot="1">
+      <c r="A25" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="B25" s="36" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>570</v>
+      </c>
+      <c r="E25" s="36">
+        <v>230</v>
+      </c>
+      <c r="F25" s="55"/>
+    </row>
+    <row r="26" spans="1:6" ht="16" thickBot="1">
+      <c r="A26" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D26" s="35" t="s">
+        <v>573</v>
+      </c>
+      <c r="E26" s="54"/>
+      <c r="F26" s="35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16" thickBot="1">
+      <c r="A27" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="C27" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E27" s="55"/>
+      <c r="F27" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16" thickBot="1">
+      <c r="A28" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="C28" s="36" t="s">
+        <v>578</v>
+      </c>
+      <c r="D28" s="36" t="s">
+        <v>579</v>
+      </c>
+      <c r="E28" s="36">
+        <v>5500</v>
+      </c>
+      <c r="F28" s="55"/>
+    </row>
+    <row r="29" spans="1:6" ht="16" thickBot="1">
+      <c r="A29" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B29" s="36" t="s">
+        <v>196</v>
+      </c>
+      <c r="C29" s="36" t="s">
+        <v>597</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E29" s="55"/>
+      <c r="F29" s="36">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16" thickBot="1">
+      <c r="A30" s="35" t="s">
+        <v>575</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="C30" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D30" s="35" t="s">
+        <v>576</v>
+      </c>
+      <c r="E30" s="54"/>
+      <c r="F30" s="35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="16" thickBot="1">
+      <c r="A31" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" s="35" t="s">
+        <v>213</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D31" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E31" s="54"/>
+      <c r="F31" s="35">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="16" thickBot="1">
+      <c r="A32" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>214</v>
+      </c>
+      <c r="C32" s="36" t="s">
+        <v>599</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>598</v>
+      </c>
+      <c r="E32" s="55"/>
+      <c r="F32" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="16" thickBot="1">
+      <c r="A33" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="C33" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E33" s="36">
+        <v>242</v>
+      </c>
+      <c r="F33" s="55"/>
+    </row>
+    <row r="34" spans="1:6" ht="16" thickBot="1">
+      <c r="A34" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>586</v>
+      </c>
+      <c r="C34" s="36" t="s">
+        <v>587</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>588</v>
+      </c>
+      <c r="E34" s="55"/>
+      <c r="F34" s="36">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="16" thickBot="1">
+      <c r="A35" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>244</v>
+      </c>
+      <c r="C35" s="35" t="s">
+        <v>600</v>
+      </c>
+      <c r="D35" s="35" t="s">
+        <v>601</v>
+      </c>
+      <c r="E35" s="54"/>
+      <c r="F35" s="35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="16" thickBot="1">
+      <c r="A36" s="35" t="s">
+        <v>170</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>265</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D36" s="35" t="s">
+        <v>576</v>
+      </c>
+      <c r="E36" s="54"/>
+      <c r="F36" s="35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="16" thickBot="1">
+      <c r="A37" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="36" t="s">
+        <v>613</v>
+      </c>
+      <c r="C37" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D37" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E37" s="36">
+        <v>50</v>
+      </c>
+      <c r="F37" s="55"/>
+    </row>
+    <row r="38" spans="1:6" ht="16" thickBot="1">
+      <c r="A38" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>624</v>
+      </c>
+      <c r="C38" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D38" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E38" s="54"/>
+      <c r="F38" s="35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16" thickBot="1">
+      <c r="A39" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>276</v>
+      </c>
+      <c r="C39" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D39" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E39" s="54"/>
+      <c r="F39" s="35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16" thickBot="1">
+      <c r="A40" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" s="36" t="s">
+        <v>568</v>
+      </c>
+      <c r="C40" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D40" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E40" s="55"/>
+      <c r="F40" s="36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16" thickBot="1">
+      <c r="A41" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B41" s="36" t="s">
+        <v>278</v>
+      </c>
+      <c r="C41" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D41" s="36" t="s">
+        <v>574</v>
+      </c>
+      <c r="E41" s="55"/>
+      <c r="F41" s="36">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16" thickBot="1">
+      <c r="A42" s="35" t="s">
+        <v>620</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>621</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>591</v>
+      </c>
+      <c r="D42" s="35" t="s">
+        <v>611</v>
+      </c>
+      <c r="E42" s="35">
+        <v>300</v>
+      </c>
+      <c r="F42" s="54"/>
+    </row>
+    <row r="43" spans="1:6" ht="16" thickBot="1">
+      <c r="A43" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B43" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C43" s="36" t="s">
+        <v>580</v>
+      </c>
+      <c r="D43" s="36" t="s">
+        <v>581</v>
+      </c>
+      <c r="E43" s="55"/>
+      <c r="F43" s="36">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16" thickBot="1">
+      <c r="A44" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C44" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D44" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E44" s="35">
+        <v>34</v>
+      </c>
+      <c r="F44" s="54"/>
+    </row>
+    <row r="45" spans="1:6" ht="16" thickBot="1">
+      <c r="A45" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>565</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>566</v>
+      </c>
+      <c r="D45" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="E45" s="54"/>
+      <c r="F45" s="35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16" thickBot="1">
+      <c r="A46" s="36" t="s">
+        <v>620</v>
+      </c>
+      <c r="B46" s="36" t="s">
+        <v>307</v>
+      </c>
+      <c r="C46" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D46" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E46" s="55"/>
+      <c r="F46" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="16" thickBot="1">
+      <c r="A47" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="36" t="s">
+        <v>308</v>
+      </c>
+      <c r="C47" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D47" s="36" t="s">
+        <v>598</v>
+      </c>
+      <c r="E47" s="55"/>
+      <c r="F47" s="36">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16" thickBot="1">
+      <c r="A48" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="36" t="s">
+        <v>312</v>
+      </c>
+      <c r="C48" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D48" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E48" s="55"/>
+      <c r="F48" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16" thickBot="1">
+      <c r="A49" s="36" t="s">
+        <v>176</v>
+      </c>
+      <c r="B49" s="36" t="s">
+        <v>316</v>
+      </c>
+      <c r="C49" s="36" t="s">
+        <v>594</v>
+      </c>
+      <c r="D49" s="36" t="s">
+        <v>589</v>
+      </c>
+      <c r="E49" s="55"/>
+      <c r="F49" s="36">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="16" thickBot="1">
+      <c r="A50" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B50" s="35" t="s">
+        <v>320</v>
+      </c>
+      <c r="C50" s="35" t="s">
+        <v>609</v>
+      </c>
+      <c r="D50" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="E50" s="54"/>
+      <c r="F50" s="35">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="16" thickBot="1">
+      <c r="A51" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" s="35" t="s">
+        <v>337</v>
+      </c>
+      <c r="C51" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D51" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E51" s="35">
+        <v>60</v>
+      </c>
+      <c r="F51" s="54"/>
+    </row>
+    <row r="52" spans="1:6" ht="16" thickBot="1">
+      <c r="A52" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B52" s="36" t="s">
+        <v>341</v>
+      </c>
+      <c r="C52" s="36" t="s">
+        <v>609</v>
+      </c>
+      <c r="D52" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E52" s="55"/>
+      <c r="F52" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="16" thickBot="1">
+      <c r="A53" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" s="36" t="s">
+        <v>342</v>
+      </c>
+      <c r="C53" s="36" t="s">
+        <v>597</v>
+      </c>
+      <c r="D53" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E53" s="55"/>
+      <c r="F53" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="16" thickBot="1">
+      <c r="A54" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B54" s="36" t="s">
+        <v>343</v>
+      </c>
+      <c r="C54" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D54" s="36" t="s">
+        <v>602</v>
+      </c>
+      <c r="E54" s="55"/>
+      <c r="F54" s="36">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="16" thickBot="1">
+      <c r="A55" s="35" t="s">
+        <v>99</v>
+      </c>
+      <c r="B55" s="35" t="s">
+        <v>352</v>
+      </c>
+      <c r="C55" s="35" t="s">
+        <v>584</v>
+      </c>
+      <c r="D55" s="35" t="s">
+        <v>585</v>
+      </c>
+      <c r="E55" s="54"/>
+      <c r="F55" s="35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="16" thickBot="1">
+      <c r="A56" s="36" t="s">
+        <v>357</v>
+      </c>
+      <c r="B56" s="36" t="s">
+        <v>358</v>
+      </c>
+      <c r="C56" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D56" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E56" s="55"/>
+      <c r="F56" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="16" thickBot="1">
+      <c r="A57" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="35" t="s">
+        <v>359</v>
+      </c>
+      <c r="C57" s="35" t="s">
+        <v>240</v>
+      </c>
+      <c r="D57" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E57" s="54"/>
+      <c r="F57" s="35">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="16" thickBot="1">
+      <c r="A58" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="36" t="s">
+        <v>363</v>
+      </c>
+      <c r="C58" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D58" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E58" s="55"/>
+      <c r="F58" s="36">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="16" thickBot="1">
+      <c r="A59" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B59" s="35" t="s">
         <v>364</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C59" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D59" s="35" t="s">
         <v>564</v>
       </c>
-      <c r="E3" s="40">
+      <c r="E59" s="35">
         <v>70</v>
       </c>
-      <c r="F3" s="41"/>
-    </row>
-    <row r="4" spans="1:7" ht="16" thickBot="1">
-      <c r="A4" s="42" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" s="44" t="s">
+      <c r="F59" s="54"/>
+    </row>
+    <row r="60" spans="1:6" ht="16" thickBot="1">
+      <c r="A60" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60" s="36" t="s">
+        <v>608</v>
+      </c>
+      <c r="C60" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D60" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E60" s="55"/>
+      <c r="F60" s="36">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="16" thickBot="1">
+      <c r="A61" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B61" s="36" t="s">
+        <v>371</v>
+      </c>
+      <c r="C61" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D61" s="36" t="s">
+        <v>567</v>
+      </c>
+      <c r="E61" s="55"/>
+      <c r="F61" s="36">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="16" thickBot="1">
+      <c r="A62" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" s="35" t="s">
+        <v>625</v>
+      </c>
+      <c r="C62" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D62" s="35" t="s">
+        <v>567</v>
+      </c>
+      <c r="E62" s="54"/>
+      <c r="F62" s="35">
+        <v>1957</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="16" thickBot="1">
+      <c r="A63" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B63" s="35" t="s">
+        <v>380</v>
+      </c>
+      <c r="C63" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D63" s="35" t="s">
+        <v>589</v>
+      </c>
+      <c r="E63" s="35">
+        <v>775</v>
+      </c>
+      <c r="F63" s="54"/>
+    </row>
+    <row r="64" spans="1:6" ht="16" thickBot="1">
+      <c r="A64" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B64" s="35" t="s">
+        <v>410</v>
+      </c>
+      <c r="C64" s="35" t="s">
+        <v>569</v>
+      </c>
+      <c r="D64" s="35" t="s">
+        <v>589</v>
+      </c>
+      <c r="E64" s="54"/>
+      <c r="F64" s="35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="16" thickBot="1">
+      <c r="A65" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="35" t="s">
+        <v>414</v>
+      </c>
+      <c r="C65" s="35" t="s">
+        <v>569</v>
+      </c>
+      <c r="D65" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="E65" s="35">
+        <v>3700</v>
+      </c>
+      <c r="F65" s="54"/>
+    </row>
+    <row r="66" spans="1:6" ht="16" thickBot="1">
+      <c r="A66" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B66" s="36" t="s">
+        <v>419</v>
+      </c>
+      <c r="C66" s="36" t="s">
+        <v>591</v>
+      </c>
+      <c r="D66" s="36" t="s">
+        <v>603</v>
+      </c>
+      <c r="E66" s="36">
+        <v>725</v>
+      </c>
+      <c r="F66" s="55"/>
+    </row>
+    <row r="67" spans="1:6" ht="16" thickBot="1">
+      <c r="A67" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B67" s="35" t="s">
+        <v>421</v>
+      </c>
+      <c r="C67" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D67" s="35" t="s">
         <v>564</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="44">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="16" thickBot="1">
-      <c r="A5" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>565</v>
-      </c>
-      <c r="C5" s="40" t="s">
-        <v>566</v>
-      </c>
-      <c r="D5" s="40" t="s">
+      <c r="E67" s="35">
+        <v>300</v>
+      </c>
+      <c r="F67" s="54"/>
+    </row>
+    <row r="68" spans="1:6" ht="16" thickBot="1">
+      <c r="A68" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B68" s="35" t="s">
+        <v>424</v>
+      </c>
+      <c r="C68" s="35" t="s">
+        <v>604</v>
+      </c>
+      <c r="D68" s="35" t="s">
+        <v>589</v>
+      </c>
+      <c r="E68" s="54"/>
+      <c r="F68" s="35">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="16" thickBot="1">
+      <c r="A69" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B69" s="36" t="s">
+        <v>425</v>
+      </c>
+      <c r="C69" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D69" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="E69" s="36">
+        <v>34</v>
+      </c>
+      <c r="F69" s="55"/>
+    </row>
+    <row r="70" spans="1:6" ht="16" thickBot="1">
+      <c r="A70" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B70" s="36" t="s">
+        <v>605</v>
+      </c>
+      <c r="C70" s="36" t="s">
+        <v>569</v>
+      </c>
+      <c r="D70" s="36" t="s">
+        <v>606</v>
+      </c>
+      <c r="E70" s="36">
+        <v>115</v>
+      </c>
+      <c r="F70" s="55"/>
+    </row>
+    <row r="71" spans="1:6" ht="16" thickBot="1">
+      <c r="A71" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B71" s="36" t="s">
+        <v>427</v>
+      </c>
+      <c r="C71" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D71" s="36" t="s">
+        <v>573</v>
+      </c>
+      <c r="E71" s="55"/>
+      <c r="F71" s="36">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="16" thickBot="1">
+      <c r="A72" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B72" s="35" t="s">
+        <v>428</v>
+      </c>
+      <c r="C72" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D72" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E72" s="35">
+        <v>110</v>
+      </c>
+      <c r="F72" s="54"/>
+    </row>
+    <row r="73" spans="1:6" ht="16" thickBot="1">
+      <c r="A73" s="35" t="s">
+        <v>357</v>
+      </c>
+      <c r="B73" s="35" t="s">
+        <v>430</v>
+      </c>
+      <c r="C73" s="35" t="s">
+        <v>584</v>
+      </c>
+      <c r="D73" s="35" t="s">
+        <v>585</v>
+      </c>
+      <c r="E73" s="54"/>
+      <c r="F73" s="35">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="16" thickBot="1">
+      <c r="A74" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B74" s="36" t="s">
+        <v>615</v>
+      </c>
+      <c r="C74" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D74" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E74" s="55"/>
+      <c r="F74" s="36">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="16" thickBot="1">
+      <c r="A75" s="35" t="s">
+        <v>616</v>
+      </c>
+      <c r="B75" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="C75" s="35" t="s">
+        <v>597</v>
+      </c>
+      <c r="D75" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="40">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="25.5" thickBot="1">
-      <c r="A6" s="42" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="43" t="s">
-        <v>568</v>
-      </c>
-      <c r="C6" s="44" t="s">
+      <c r="E75" s="54"/>
+      <c r="F75" s="35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="16" thickBot="1">
+      <c r="A76" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="B76" s="35" t="s">
+        <v>436</v>
+      </c>
+      <c r="C76" s="35" t="s">
+        <v>594</v>
+      </c>
+      <c r="D76" s="35" t="s">
+        <v>619</v>
+      </c>
+      <c r="E76" s="54"/>
+      <c r="F76" s="35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="16" thickBot="1">
+      <c r="A77" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="B77" s="35" t="s">
+        <v>582</v>
+      </c>
+      <c r="C77" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="D6" s="44" t="s">
+      <c r="D77" s="35" t="s">
+        <v>583</v>
+      </c>
+      <c r="E77" s="54"/>
+      <c r="F77" s="35">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="16" thickBot="1">
+      <c r="A78" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B78" s="36" t="s">
+        <v>441</v>
+      </c>
+      <c r="C78" s="36" t="s">
+        <v>584</v>
+      </c>
+      <c r="D78" s="36" t="s">
+        <v>573</v>
+      </c>
+      <c r="E78" s="36">
+        <v>147</v>
+      </c>
+      <c r="F78" s="55"/>
+    </row>
+    <row r="79" spans="1:6" ht="16" thickBot="1">
+      <c r="A79" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B79" s="35" t="s">
+        <v>444</v>
+      </c>
+      <c r="C79" s="35" t="s">
+        <v>600</v>
+      </c>
+      <c r="D79" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E79" s="54"/>
+      <c r="F79" s="54"/>
+    </row>
+    <row r="80" spans="1:6" ht="16" thickBot="1">
+      <c r="A80" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B80" s="36" t="s">
+        <v>448</v>
+      </c>
+      <c r="C80" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D80" s="36" t="s">
+        <v>574</v>
+      </c>
+      <c r="E80" s="55"/>
+      <c r="F80" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="16" thickBot="1">
+      <c r="A81" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B81" s="35" t="s">
+        <v>610</v>
+      </c>
+      <c r="C81" s="35" t="s">
+        <v>584</v>
+      </c>
+      <c r="D81" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E6" s="45"/>
-      <c r="F6" s="44">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="16" thickBot="1">
-      <c r="A7" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>414</v>
-      </c>
-      <c r="C7" s="40" t="s">
-        <v>569</v>
-      </c>
-      <c r="D7" s="39" t="s">
-        <v>570</v>
-      </c>
-      <c r="E7" s="40">
-        <v>3700</v>
-      </c>
-      <c r="F7" s="41"/>
-    </row>
-    <row r="8" spans="1:7" ht="16" thickBot="1">
-      <c r="A8" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="44" t="s">
+      <c r="E81" s="54"/>
+      <c r="F81" s="35">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="16" thickBot="1">
+      <c r="A82" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" s="35" t="s">
+        <v>459</v>
+      </c>
+      <c r="C82" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D82" s="35" t="s">
+        <v>598</v>
+      </c>
+      <c r="E82" s="54"/>
+      <c r="F82" s="35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="16" thickBot="1">
+      <c r="A83" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="B83" s="35" t="s">
+        <v>461</v>
+      </c>
+      <c r="C83" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D83" s="35" t="s">
+        <v>614</v>
+      </c>
+      <c r="E83" s="35">
+        <v>640</v>
+      </c>
+      <c r="F83" s="54"/>
+    </row>
+    <row r="84" spans="1:6" ht="16" thickBot="1">
+      <c r="A84" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B84" s="35" t="s">
+        <v>490</v>
+      </c>
+      <c r="C84" s="35" t="s">
+        <v>584</v>
+      </c>
+      <c r="D84" s="35" t="s">
+        <v>607</v>
+      </c>
+      <c r="E84" s="35">
+        <v>78</v>
+      </c>
+      <c r="F84" s="54"/>
+    </row>
+    <row r="85" spans="1:6" ht="16" thickBot="1">
+      <c r="A85" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B85" s="36" t="s">
+        <v>512</v>
+      </c>
+      <c r="C85" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="D85" s="36" t="s">
         <v>564</v>
       </c>
-      <c r="E8" s="44">
-        <v>2</v>
-      </c>
-      <c r="F8" s="45"/>
-    </row>
-    <row r="9" spans="1:7" ht="16" thickBot="1">
-      <c r="A9" s="38" t="s">
+      <c r="E85" s="55"/>
+      <c r="F85" s="36">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="16" thickBot="1">
+      <c r="A86" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="B86" s="36" t="s">
+        <v>514</v>
+      </c>
+      <c r="C86" s="36" t="s">
+        <v>591</v>
+      </c>
+      <c r="D86" s="36" t="s">
+        <v>589</v>
+      </c>
+      <c r="E86" s="36">
+        <v>2625</v>
+      </c>
+      <c r="F86" s="55"/>
+    </row>
+    <row r="87" spans="1:6" ht="16" thickBot="1">
+      <c r="A87" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="B87" s="35" t="s">
+        <v>526</v>
+      </c>
+      <c r="C87" s="35" t="s">
+        <v>563</v>
+      </c>
+      <c r="D87" s="35" t="s">
+        <v>564</v>
+      </c>
+      <c r="E87" s="54"/>
+      <c r="F87" s="35">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="16" thickBot="1">
+      <c r="A88" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="39" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="40" t="s">
+      <c r="B88" s="35" t="s">
+        <v>528</v>
+      </c>
+      <c r="C88" s="35" t="s">
         <v>563</v>
       </c>
-      <c r="D9" s="39" t="s">
-        <v>564</v>
-      </c>
-      <c r="E9" s="40">
-        <v>115</v>
-      </c>
-      <c r="F9" s="41"/>
-    </row>
-    <row r="10" spans="1:7" ht="16" thickBot="1">
-      <c r="A10" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D10" s="43" t="s">
-        <v>564</v>
-      </c>
-      <c r="E10" s="44">
-        <v>56</v>
-      </c>
-      <c r="F10" s="45"/>
-    </row>
-    <row r="11" spans="1:7" ht="16" thickBot="1">
-      <c r="A11" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="39" t="s">
-        <v>571</v>
-      </c>
-      <c r="C11" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D11" s="39" t="s">
-        <v>572</v>
-      </c>
-      <c r="E11" s="40">
-        <v>1300</v>
-      </c>
-      <c r="F11" s="41"/>
-    </row>
-    <row r="12" spans="1:7" ht="16" thickBot="1">
-      <c r="A12" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>122</v>
-      </c>
-      <c r="C12" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D12" s="43" t="s">
-        <v>564</v>
-      </c>
-      <c r="E12" s="44">
-        <v>1</v>
-      </c>
-      <c r="F12" s="45"/>
-    </row>
-    <row r="13" spans="1:7" ht="16" thickBot="1">
-      <c r="A13" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="C13" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D13" s="39" t="s">
+      <c r="D88" s="35" t="s">
         <v>573</v>
       </c>
-      <c r="E13" s="41"/>
-      <c r="F13" s="40">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="16" thickBot="1">
-      <c r="A14" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="43" t="s">
-        <v>278</v>
-      </c>
-      <c r="C14" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D14" s="43" t="s">
-        <v>574</v>
-      </c>
-      <c r="E14" s="45"/>
-      <c r="F14" s="44">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="16" thickBot="1">
-      <c r="A15" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="39" t="s">
-        <v>294</v>
-      </c>
-      <c r="C15" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D15" s="39" t="s">
-        <v>564</v>
-      </c>
-      <c r="E15" s="40">
-        <v>34</v>
-      </c>
-      <c r="F15" s="41"/>
-    </row>
-    <row r="16" spans="1:7" ht="16" thickBot="1">
-      <c r="A16" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="43" t="s">
-        <v>427</v>
-      </c>
-      <c r="C16" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D16" s="43" t="s">
-        <v>573</v>
-      </c>
-      <c r="E16" s="45"/>
-      <c r="F16" s="44">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="16" thickBot="1">
-      <c r="A17" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="39" t="s">
-        <v>428</v>
-      </c>
-      <c r="C17" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D17" s="39" t="s">
-        <v>564</v>
-      </c>
-      <c r="E17" s="40">
-        <v>110</v>
-      </c>
-      <c r="F17" s="41"/>
-    </row>
-    <row r="18" spans="1:6" ht="16" thickBot="1">
-      <c r="A18" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>448</v>
-      </c>
-      <c r="C18" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D18" s="43" t="s">
-        <v>574</v>
-      </c>
-      <c r="E18" s="45"/>
-      <c r="F18" s="44">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="16" thickBot="1">
-      <c r="A19" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="39" t="s">
-        <v>528</v>
-      </c>
-      <c r="C19" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D19" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="E19" s="41"/>
-      <c r="F19" s="40">
+      <c r="E88" s="54"/>
+      <c r="F88" s="35">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="16" thickBot="1">
-      <c r="A20" s="42" t="s">
-        <v>188</v>
-      </c>
-      <c r="B20" s="43" t="s">
-        <v>189</v>
-      </c>
-      <c r="C20" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D20" s="43" t="s">
-        <v>570</v>
-      </c>
-      <c r="E20" s="44">
-        <v>230</v>
-      </c>
-      <c r="F20" s="45"/>
-    </row>
-    <row r="21" spans="1:6" ht="16" thickBot="1">
-      <c r="A21" s="38" t="s">
-        <v>575</v>
-      </c>
-      <c r="B21" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="C21" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D21" s="39" t="s">
-        <v>576</v>
-      </c>
-      <c r="E21" s="41"/>
-      <c r="F21" s="40">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="16" thickBot="1">
-      <c r="A22" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="B22" s="44" t="s">
-        <v>171</v>
-      </c>
-      <c r="C22" s="43" t="s">
-        <v>563</v>
-      </c>
-      <c r="D22" s="43" t="s">
-        <v>577</v>
-      </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="44">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="16" thickBot="1">
-      <c r="A23" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="B23" s="39" t="s">
-        <v>265</v>
-      </c>
-      <c r="C23" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D23" s="39" t="s">
-        <v>576</v>
-      </c>
-      <c r="E23" s="41"/>
-      <c r="F23" s="40">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="16" thickBot="1">
-      <c r="A24" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="B24" s="43" t="s">
-        <v>425</v>
-      </c>
-      <c r="C24" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D24" s="43" t="s">
-        <v>564</v>
-      </c>
-      <c r="E24" s="44">
-        <v>34</v>
-      </c>
-      <c r="F24" s="45"/>
-    </row>
-    <row r="25" spans="1:6" ht="16" thickBot="1">
-      <c r="A25" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D25" s="39" t="s">
-        <v>570</v>
-      </c>
-      <c r="E25" s="46">
-        <v>3475</v>
-      </c>
-      <c r="F25" s="41"/>
-    </row>
-    <row r="26" spans="1:6" ht="16" thickBot="1">
-      <c r="A26" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="B26" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="C26" s="44" t="s">
-        <v>578</v>
-      </c>
-      <c r="D26" s="43" t="s">
-        <v>579</v>
-      </c>
-      <c r="E26" s="44">
-        <v>5500</v>
-      </c>
-      <c r="F26" s="45"/>
-    </row>
-    <row r="27" spans="1:6" ht="16" thickBot="1">
-      <c r="A27" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="39" t="s">
-        <v>276</v>
-      </c>
-      <c r="C27" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D27" s="39" t="s">
-        <v>564</v>
-      </c>
-      <c r="E27" s="41"/>
-      <c r="F27" s="40">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="16" thickBot="1">
-      <c r="A28" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>293</v>
-      </c>
-      <c r="C28" s="44" t="s">
-        <v>580</v>
-      </c>
-      <c r="D28" s="43" t="s">
-        <v>581</v>
-      </c>
-      <c r="E28" s="45"/>
-      <c r="F28" s="44">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A29" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>582</v>
-      </c>
-      <c r="C29" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D29" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="E29" s="41"/>
-      <c r="F29" s="40">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="16" thickBot="1">
-      <c r="A30" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="B30" s="43" t="s">
-        <v>512</v>
-      </c>
-      <c r="C30" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D30" s="43" t="s">
-        <v>564</v>
-      </c>
-      <c r="E30" s="45"/>
-      <c r="F30" s="44">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="16" thickBot="1">
-      <c r="A31" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="B31" s="39" t="s">
-        <v>526</v>
-      </c>
-      <c r="C31" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D31" s="39" t="s">
-        <v>564</v>
-      </c>
-      <c r="E31" s="41"/>
-      <c r="F31" s="40">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="16" thickBot="1">
-      <c r="A32" s="42" t="s">
-        <v>357</v>
-      </c>
-      <c r="B32" s="43" t="s">
-        <v>358</v>
-      </c>
-      <c r="C32" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D32" s="43" t="s">
-        <v>564</v>
-      </c>
-      <c r="E32" s="45"/>
-      <c r="F32" s="44">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="16" thickBot="1">
-      <c r="A33" s="38" t="s">
-        <v>357</v>
-      </c>
-      <c r="B33" s="39" t="s">
-        <v>430</v>
-      </c>
-      <c r="C33" s="40" t="s">
-        <v>584</v>
-      </c>
-      <c r="D33" s="40" t="s">
-        <v>585</v>
-      </c>
-      <c r="E33" s="41"/>
-      <c r="F33" s="40">
-        <v>1660</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A34" s="42" t="s">
-        <v>236</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>586</v>
-      </c>
-      <c r="C34" s="44" t="s">
-        <v>587</v>
-      </c>
-      <c r="D34" s="44" t="s">
-        <v>588</v>
-      </c>
-      <c r="E34" s="45"/>
-      <c r="F34" s="44">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="16" thickBot="1">
-      <c r="A35" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="B35" s="39" t="s">
-        <v>380</v>
-      </c>
-      <c r="C35" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D35" s="40" t="s">
-        <v>589</v>
-      </c>
-      <c r="E35" s="40">
-        <v>775</v>
-      </c>
-      <c r="F35" s="41"/>
-    </row>
-    <row r="36" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A36" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B36" s="43" t="s">
-        <v>590</v>
-      </c>
-      <c r="C36" s="43" t="s">
+    <row r="89" spans="1:6">
+      <c r="A89" s="34" t="s">
+        <v>298</v>
+      </c>
+      <c r="B89" s="34" t="s">
+        <v>529</v>
+      </c>
+      <c r="C89" s="34" t="s">
         <v>591</v>
       </c>
-      <c r="D36" s="43" t="s">
+      <c r="D89" s="34" t="s">
         <v>592</v>
       </c>
-      <c r="E36" s="45"/>
-      <c r="F36" s="44">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="16" thickBot="1">
-      <c r="A37" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="B37" s="40" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37" s="39" t="s">
-        <v>563</v>
-      </c>
-      <c r="D37" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E37" s="41"/>
-      <c r="F37" s="40">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A38" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B38" s="43" t="s">
-        <v>593</v>
-      </c>
-      <c r="C38" s="44" t="s">
-        <v>594</v>
-      </c>
-      <c r="D38" s="43" t="s">
-        <v>595</v>
-      </c>
-      <c r="E38" s="45"/>
-      <c r="F38" s="44">
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="16" thickBot="1">
-      <c r="A39" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="C39" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D39" s="40" t="s">
-        <v>596</v>
-      </c>
-      <c r="E39" s="41"/>
-      <c r="F39" s="40">
-        <v>2625</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="16" thickBot="1">
-      <c r="A40" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B40" s="44" t="s">
-        <v>196</v>
-      </c>
-      <c r="C40" s="44" t="s">
-        <v>597</v>
-      </c>
-      <c r="D40" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E40" s="45"/>
-      <c r="F40" s="44">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="16" thickBot="1">
-      <c r="A41" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" s="39" t="s">
-        <v>213</v>
-      </c>
-      <c r="C41" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D41" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E41" s="41"/>
-      <c r="F41" s="40">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="16" thickBot="1">
-      <c r="A42" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>214</v>
-      </c>
-      <c r="C42" s="44" t="s">
-        <v>599</v>
-      </c>
-      <c r="D42" s="44" t="s">
-        <v>598</v>
-      </c>
-      <c r="E42" s="45"/>
-      <c r="F42" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="16" thickBot="1">
-      <c r="A43" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B43" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="C43" s="40" t="s">
-        <v>600</v>
-      </c>
-      <c r="D43" s="40" t="s">
-        <v>601</v>
-      </c>
-      <c r="E43" s="41"/>
-      <c r="F43" s="40">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="16" thickBot="1">
-      <c r="A44" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B44" s="43" t="s">
-        <v>343</v>
-      </c>
-      <c r="C44" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D44" s="44" t="s">
-        <v>602</v>
-      </c>
-      <c r="E44" s="45"/>
-      <c r="F44" s="44">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="16" thickBot="1">
-      <c r="A45" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B45" s="39" t="s">
-        <v>359</v>
-      </c>
-      <c r="C45" s="40" t="s">
-        <v>240</v>
-      </c>
-      <c r="D45" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E45" s="41"/>
-      <c r="F45" s="40">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="16" thickBot="1">
-      <c r="A46" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="43" t="s">
-        <v>363</v>
-      </c>
-      <c r="C46" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D46" s="44" t="s">
-        <v>227</v>
-      </c>
-      <c r="E46" s="45"/>
-      <c r="F46" s="44">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="16" thickBot="1">
-      <c r="A47" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B47" s="39" t="s">
-        <v>410</v>
-      </c>
-      <c r="C47" s="40" t="s">
-        <v>569</v>
-      </c>
-      <c r="D47" s="40" t="s">
-        <v>589</v>
-      </c>
-      <c r="E47" s="41"/>
-      <c r="F47" s="40">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="16" thickBot="1">
-      <c r="A48" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B48" s="43" t="s">
-        <v>419</v>
-      </c>
-      <c r="C48" s="44" t="s">
-        <v>591</v>
-      </c>
-      <c r="D48" s="44" t="s">
-        <v>603</v>
-      </c>
-      <c r="E48" s="44">
-        <v>725</v>
-      </c>
-      <c r="F48" s="45"/>
-    </row>
-    <row r="49" spans="1:6" ht="16" thickBot="1">
-      <c r="A49" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B49" s="39" t="s">
-        <v>424</v>
-      </c>
-      <c r="C49" s="40" t="s">
-        <v>604</v>
-      </c>
-      <c r="D49" s="40" t="s">
-        <v>589</v>
-      </c>
-      <c r="E49" s="41"/>
-      <c r="F49" s="40">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="16" thickBot="1">
-      <c r="A50" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B50" s="43" t="s">
-        <v>605</v>
-      </c>
-      <c r="C50" s="44" t="s">
-        <v>569</v>
-      </c>
-      <c r="D50" s="44" t="s">
-        <v>606</v>
-      </c>
-      <c r="E50" s="44">
-        <v>115</v>
-      </c>
-      <c r="F50" s="45"/>
-    </row>
-    <row r="51" spans="1:6" ht="16" thickBot="1">
-      <c r="A51" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B51" s="39" t="s">
-        <v>490</v>
-      </c>
-      <c r="C51" s="40" t="s">
-        <v>584</v>
-      </c>
-      <c r="D51" s="40" t="s">
-        <v>607</v>
-      </c>
-      <c r="E51" s="40">
-        <v>78</v>
-      </c>
-      <c r="F51" s="41"/>
-    </row>
-    <row r="52" spans="1:6" ht="16" thickBot="1">
-      <c r="A52" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="B52" s="43" t="s">
-        <v>608</v>
-      </c>
-      <c r="C52" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D52" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E52" s="45"/>
-      <c r="F52" s="44">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="16" thickBot="1">
-      <c r="A53" s="38" t="s">
-        <v>87</v>
-      </c>
-      <c r="B53" s="40" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D53" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E53" s="41"/>
-      <c r="F53" s="40">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="16" thickBot="1">
-      <c r="A54" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="B54" s="43" t="s">
-        <v>371</v>
-      </c>
-      <c r="C54" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D54" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E54" s="45"/>
-      <c r="F54" s="44">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="16" thickBot="1">
-      <c r="A55" s="38" t="s">
-        <v>87</v>
-      </c>
-      <c r="B55" s="39" t="s">
-        <v>320</v>
-      </c>
-      <c r="C55" s="40" t="s">
-        <v>609</v>
-      </c>
-      <c r="D55" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E55" s="41"/>
-      <c r="F55" s="40">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="16" thickBot="1">
-      <c r="A56" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="B56" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="C56" s="44" t="s">
-        <v>609</v>
-      </c>
-      <c r="D56" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E56" s="45"/>
-      <c r="F56" s="44">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="16" thickBot="1">
-      <c r="A57" s="38" t="s">
-        <v>87</v>
-      </c>
-      <c r="B57" s="39" t="s">
-        <v>610</v>
-      </c>
-      <c r="C57" s="40" t="s">
-        <v>584</v>
-      </c>
-      <c r="D57" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E57" s="41"/>
-      <c r="F57" s="40">
-        <v>1097</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="16" thickBot="1">
-      <c r="A58" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="44" t="s">
-        <v>193</v>
-      </c>
-      <c r="C58" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D58" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E58" s="45"/>
-      <c r="F58" s="44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="16" thickBot="1">
-      <c r="A59" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="B59" s="39" t="s">
-        <v>181</v>
-      </c>
-      <c r="C59" s="40" t="s">
-        <v>594</v>
-      </c>
-      <c r="D59" s="39" t="s">
-        <v>611</v>
-      </c>
-      <c r="E59" s="40" t="s">
-        <v>612</v>
-      </c>
-      <c r="F59" s="40">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="16" thickBot="1">
-      <c r="A60" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="B60" s="43" t="s">
-        <v>613</v>
-      </c>
-      <c r="C60" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D60" s="44" t="s">
-        <v>564</v>
-      </c>
-      <c r="E60" s="44">
-        <v>50</v>
-      </c>
-      <c r="F60" s="45"/>
-    </row>
-    <row r="61" spans="1:6" ht="16" thickBot="1">
-      <c r="A61" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="39" t="s">
-        <v>461</v>
-      </c>
-      <c r="C61" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D61" s="40" t="s">
-        <v>614</v>
-      </c>
-      <c r="E61" s="40">
-        <v>640</v>
-      </c>
-      <c r="F61" s="41"/>
-    </row>
-    <row r="62" spans="1:6" ht="16" thickBot="1">
-      <c r="A62" s="42" t="s">
-        <v>298</v>
-      </c>
-      <c r="B62" s="43" t="s">
-        <v>529</v>
-      </c>
-      <c r="C62" s="43" t="s">
-        <v>591</v>
-      </c>
-      <c r="D62" s="44" t="s">
-        <v>592</v>
-      </c>
-      <c r="E62" s="44">
+      <c r="E89" s="34">
         <v>285</v>
       </c>
-      <c r="F62" s="45"/>
-    </row>
-    <row r="63" spans="1:6" ht="16" thickBot="1">
-      <c r="A63" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="B63" s="39" t="s">
-        <v>352</v>
-      </c>
-      <c r="C63" s="40" t="s">
-        <v>584</v>
-      </c>
-      <c r="D63" s="40" t="s">
-        <v>585</v>
-      </c>
-      <c r="E63" s="41"/>
-      <c r="F63" s="40">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="16" thickBot="1">
-      <c r="A64" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="B64" s="43" t="s">
-        <v>226</v>
-      </c>
-      <c r="C64" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D64" s="44" t="s">
-        <v>227</v>
-      </c>
-      <c r="E64" s="44">
-        <v>242</v>
-      </c>
-      <c r="F64" s="45"/>
-    </row>
-    <row r="65" spans="1:6" ht="16" thickBot="1">
-      <c r="A65" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="B65" s="39" t="s">
-        <v>421</v>
-      </c>
-      <c r="C65" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D65" s="40" t="s">
-        <v>564</v>
-      </c>
-      <c r="E65" s="40">
-        <v>300</v>
-      </c>
-      <c r="F65" s="41"/>
-    </row>
-    <row r="66" spans="1:6" ht="16" thickBot="1">
-      <c r="A66" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="B66" s="43" t="s">
-        <v>615</v>
-      </c>
-      <c r="C66" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D66" s="44" t="s">
-        <v>227</v>
-      </c>
-      <c r="E66" s="45"/>
-      <c r="F66" s="44">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="16" thickBot="1">
-      <c r="A67" s="38" t="s">
-        <v>616</v>
-      </c>
-      <c r="B67" s="40" t="s">
-        <v>433</v>
-      </c>
-      <c r="C67" s="40" t="s">
-        <v>597</v>
-      </c>
-      <c r="D67" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E67" s="41"/>
-      <c r="F67" s="40">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="16" thickBot="1">
-      <c r="A68" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="B68" s="43" t="s">
-        <v>441</v>
-      </c>
-      <c r="C68" s="44" t="s">
-        <v>584</v>
-      </c>
-      <c r="D68" s="44" t="s">
-        <v>573</v>
-      </c>
-      <c r="E68" s="44">
-        <v>147</v>
-      </c>
-      <c r="F68" s="45"/>
-    </row>
-    <row r="69" spans="1:6" ht="16" thickBot="1">
-      <c r="A69" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="B69" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="C69" s="40" t="s">
-        <v>599</v>
-      </c>
-      <c r="D69" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E69" s="41"/>
-      <c r="F69" s="40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="16" thickBot="1">
-      <c r="A70" s="42" t="s">
-        <v>91</v>
-      </c>
-      <c r="B70" s="43" t="s">
-        <v>514</v>
-      </c>
-      <c r="C70" s="44" t="s">
-        <v>591</v>
-      </c>
-      <c r="D70" s="44" t="s">
-        <v>589</v>
-      </c>
-      <c r="E70" s="44">
-        <v>2625</v>
-      </c>
-      <c r="F70" s="45"/>
-    </row>
-    <row r="71" spans="1:6" ht="16" thickBot="1">
-      <c r="A71" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B71" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="C71" s="39" t="s">
-        <v>563</v>
-      </c>
-      <c r="D71" s="40" t="s">
-        <v>617</v>
-      </c>
-      <c r="E71" s="41"/>
-      <c r="F71" s="40">
-        <v>3628</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="16" thickBot="1">
-      <c r="A72" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="B72" s="43" t="s">
-        <v>141</v>
-      </c>
-      <c r="C72" s="44" t="s">
-        <v>587</v>
-      </c>
-      <c r="D72" s="44" t="s">
-        <v>618</v>
-      </c>
-      <c r="E72" s="45"/>
-      <c r="F72" s="44">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="16" thickBot="1">
-      <c r="A73" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B73" s="39" t="s">
-        <v>164</v>
-      </c>
-      <c r="C73" s="40" t="s">
-        <v>594</v>
-      </c>
-      <c r="D73" s="40" t="s">
-        <v>592</v>
-      </c>
-      <c r="E73" s="41"/>
-      <c r="F73" s="40">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="16" thickBot="1">
-      <c r="A74" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="B74" s="43" t="s">
-        <v>312</v>
-      </c>
-      <c r="C74" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D74" s="44" t="s">
-        <v>564</v>
-      </c>
-      <c r="E74" s="45"/>
-      <c r="F74" s="44">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="16" thickBot="1">
-      <c r="A75" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B75" s="39" t="s">
-        <v>436</v>
-      </c>
-      <c r="C75" s="40" t="s">
-        <v>594</v>
-      </c>
-      <c r="D75" s="40" t="s">
-        <v>619</v>
-      </c>
-      <c r="E75" s="41"/>
-      <c r="F75" s="40">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="16" thickBot="1">
-      <c r="A76" s="42" t="s">
-        <v>176</v>
-      </c>
-      <c r="B76" s="43" t="s">
-        <v>316</v>
-      </c>
-      <c r="C76" s="44" t="s">
-        <v>594</v>
-      </c>
-      <c r="D76" s="44" t="s">
-        <v>589</v>
-      </c>
-      <c r="E76" s="45"/>
-      <c r="F76" s="44">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="16" thickBot="1">
-      <c r="A77" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="B77" s="40" t="s">
-        <v>444</v>
-      </c>
-      <c r="C77" s="39" t="s">
-        <v>600</v>
-      </c>
-      <c r="D77" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E77" s="41"/>
-      <c r="F77" s="41"/>
-    </row>
-    <row r="78" spans="1:6" ht="16" thickBot="1">
-      <c r="A78" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B78" s="44" t="s">
-        <v>342</v>
-      </c>
-      <c r="C78" s="44" t="s">
-        <v>597</v>
-      </c>
-      <c r="D78" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E78" s="45"/>
-      <c r="F78" s="44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="16" thickBot="1">
-      <c r="A79" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="B79" s="40" t="s">
-        <v>459</v>
-      </c>
-      <c r="C79" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D79" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E79" s="41"/>
-      <c r="F79" s="40">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="16" thickBot="1">
-      <c r="A80" s="42" t="s">
-        <v>620</v>
-      </c>
-      <c r="B80" s="43" t="s">
-        <v>307</v>
-      </c>
-      <c r="C80" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D80" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E80" s="45"/>
-      <c r="F80" s="44">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A81" s="38" t="s">
-        <v>620</v>
-      </c>
-      <c r="B81" s="39" t="s">
-        <v>621</v>
-      </c>
-      <c r="C81" s="39" t="s">
-        <v>591</v>
-      </c>
-      <c r="D81" s="40" t="s">
-        <v>611</v>
-      </c>
-      <c r="E81" s="40">
-        <v>300</v>
-      </c>
-      <c r="F81" s="41"/>
-    </row>
-    <row r="82" spans="1:6" ht="16" thickBot="1">
-      <c r="A82" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="B82" s="43" t="s">
-        <v>622</v>
-      </c>
-      <c r="C82" s="44" t="s">
-        <v>101</v>
-      </c>
-      <c r="D82" s="44" t="s">
-        <v>573</v>
-      </c>
-      <c r="E82" s="45"/>
-      <c r="F82" s="44">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="16" thickBot="1">
-      <c r="A83" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="B83" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="C83" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D83" s="40" t="s">
-        <v>598</v>
-      </c>
-      <c r="E83" s="41"/>
-      <c r="F83" s="40">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A84" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="B84" s="43" t="s">
-        <v>623</v>
-      </c>
-      <c r="C84" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D84" s="44" t="s">
-        <v>573</v>
-      </c>
-      <c r="E84" s="44">
-        <v>75</v>
-      </c>
-      <c r="F84" s="45"/>
-    </row>
-    <row r="85" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A85" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="B85" s="39" t="s">
-        <v>624</v>
-      </c>
-      <c r="C85" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D85" s="40" t="s">
-        <v>564</v>
-      </c>
-      <c r="E85" s="41"/>
-      <c r="F85" s="40">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="16" thickBot="1">
-      <c r="A86" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="B86" s="43" t="s">
-        <v>308</v>
-      </c>
-      <c r="C86" s="44" t="s">
-        <v>563</v>
-      </c>
-      <c r="D86" s="44" t="s">
-        <v>598</v>
-      </c>
-      <c r="E86" s="45"/>
-      <c r="F86" s="44">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="25.5" thickBot="1">
-      <c r="A87" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="B87" s="39" t="s">
-        <v>625</v>
-      </c>
-      <c r="C87" s="40" t="s">
-        <v>563</v>
-      </c>
-      <c r="D87" s="40" t="s">
-        <v>567</v>
-      </c>
-      <c r="E87" s="41"/>
-      <c r="F87" s="40">
-        <v>1957</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="16" thickBot="1">
-      <c r="A88" s="42" t="s">
-        <v>173</v>
-      </c>
-      <c r="B88" s="43" t="s">
-        <v>626</v>
-      </c>
-      <c r="C88" s="43" t="s">
-        <v>240</v>
-      </c>
-      <c r="D88" s="44" t="s">
-        <v>567</v>
-      </c>
-      <c r="E88" s="45"/>
-      <c r="F88" s="44">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="16" thickBot="1">
-      <c r="A89" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="B89" s="40" t="s">
-        <v>337</v>
-      </c>
-      <c r="C89" s="39" t="s">
-        <v>563</v>
-      </c>
-      <c r="D89" s="40" t="s">
-        <v>564</v>
-      </c>
-      <c r="E89" s="40">
-        <v>60</v>
-      </c>
-      <c r="F89" s="41"/>
+      <c r="F89" s="57"/>
     </row>
     <row r="90" spans="1:6">
-      <c r="A90" s="48" t="s">
+      <c r="A90" s="37" t="s">
         <v>627</v>
       </c>
-      <c r="B90" s="49"/>
-      <c r="C90" s="50"/>
-      <c r="D90" s="49"/>
-      <c r="E90" s="51">
+      <c r="B90" s="38"/>
+      <c r="C90" s="39"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="40">
         <v>21044</v>
       </c>
-      <c r="F90" s="51">
+      <c r="F90" s="40">
         <v>24814</v>
       </c>
     </row>
@@ -17204,6 +17242,9 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -17220,10 +17261,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34" customHeight="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="45" t="s">
         <v>628</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="41" t="s">
         <v>1256</v>
       </c>
     </row>
@@ -17928,13 +17969,13 @@
       <c r="B58" s="8" t="s">
         <v>726</v>
       </c>
-      <c r="C58" s="53" t="s">
+      <c r="C58" s="41" t="s">
         <v>727</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>728</v>
       </c>
-      <c r="E58" s="53" t="s">
+      <c r="E58" s="41" t="s">
         <v>1214</v>
       </c>
     </row>
@@ -18061,13 +18102,13 @@
       <c r="B69" s="8">
         <v>78</v>
       </c>
-      <c r="C69" s="53" t="s">
+      <c r="C69" s="41" t="s">
         <v>755</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="E69" s="53" t="s">
+      <c r="E69" s="41" t="s">
         <v>794</v>
       </c>
     </row>
@@ -18162,13 +18203,13 @@
       <c r="B76" s="8">
         <v>12</v>
       </c>
-      <c r="C76" s="53" t="s">
+      <c r="C76" s="41" t="s">
         <v>739</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="E76" s="53"/>
+      <c r="E76" s="41"/>
     </row>
     <row r="77" spans="1:5" s="8" customFormat="1" ht="46.5">
       <c r="A77" s="8" t="s">
@@ -18177,13 +18218,13 @@
       <c r="B77" s="8">
         <v>37</v>
       </c>
-      <c r="C77" s="53" t="s">
+      <c r="C77" s="41" t="s">
         <v>791</v>
       </c>
       <c r="D77" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="E77" s="53" t="s">
+      <c r="E77" s="41" t="s">
         <v>792</v>
       </c>
     </row>
@@ -18352,13 +18393,13 @@
       <c r="B91" s="8">
         <v>1</v>
       </c>
-      <c r="C91" s="53" t="s">
+      <c r="C91" s="41" t="s">
         <v>795</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="E91" s="53" t="s">
+      <c r="E91" s="41" t="s">
         <v>1258</v>
       </c>
     </row>
@@ -19533,13 +19574,13 @@
       </c>
     </row>
     <row r="189" spans="1:5" ht="31">
-      <c r="A189" s="54" t="s">
+      <c r="A189" s="42" t="s">
         <v>1259</v>
       </c>
       <c r="B189" s="8"/>
-      <c r="C189" s="53"/>
+      <c r="C189" s="41"/>
       <c r="D189" s="8"/>
-      <c r="E189" s="53" t="s">
+      <c r="E189" s="41" t="s">
         <v>963</v>
       </c>
     </row>
@@ -19550,11 +19591,11 @@
       <c r="B190" s="8">
         <v>1</v>
       </c>
-      <c r="C190" s="53"/>
+      <c r="C190" s="41"/>
       <c r="D190" s="8" t="s">
         <v>931</v>
       </c>
-      <c r="E190" s="53" t="s">
+      <c r="E190" s="41" t="s">
         <v>1218</v>
       </c>
     </row>
@@ -19565,7 +19606,7 @@
       <c r="B191" s="8">
         <v>4</v>
       </c>
-      <c r="C191" s="53"/>
+      <c r="C191" s="41"/>
       <c r="D191" s="8" t="s">
         <v>931</v>
       </c>
@@ -19577,7 +19618,7 @@
       <c r="B192" s="8">
         <v>4</v>
       </c>
-      <c r="C192" s="53"/>
+      <c r="C192" s="41"/>
       <c r="D192" s="8" t="s">
         <v>934</v>
       </c>
@@ -19589,7 +19630,7 @@
       <c r="B193" s="8">
         <v>2</v>
       </c>
-      <c r="C193" s="53"/>
+      <c r="C193" s="41"/>
       <c r="D193" s="8" t="s">
         <v>931</v>
       </c>
@@ -19601,7 +19642,7 @@
       <c r="B194" s="8">
         <v>8</v>
       </c>
-      <c r="C194" s="53"/>
+      <c r="C194" s="41"/>
       <c r="D194" s="8" t="s">
         <v>937</v>
       </c>
@@ -19613,7 +19654,7 @@
       <c r="B195" s="8">
         <v>3</v>
       </c>
-      <c r="C195" s="53"/>
+      <c r="C195" s="41"/>
       <c r="D195" s="8" t="s">
         <v>931</v>
       </c>
@@ -19625,7 +19666,7 @@
       <c r="B196" s="8">
         <v>19</v>
       </c>
-      <c r="C196" s="53" t="s">
+      <c r="C196" s="41" t="s">
         <v>940</v>
       </c>
       <c r="D196" s="8" t="s">
@@ -19639,7 +19680,7 @@
       <c r="B197" s="8">
         <v>1</v>
       </c>
-      <c r="C197" s="53"/>
+      <c r="C197" s="41"/>
       <c r="D197" s="8" t="s">
         <v>931</v>
       </c>
@@ -19651,7 +19692,7 @@
       <c r="B198" s="8">
         <v>6</v>
       </c>
-      <c r="C198" s="53"/>
+      <c r="C198" s="41"/>
       <c r="D198" s="8" t="s">
         <v>934</v>
       </c>
@@ -19663,7 +19704,7 @@
       <c r="B199" s="8">
         <v>1</v>
       </c>
-      <c r="C199" s="53"/>
+      <c r="C199" s="41"/>
       <c r="D199" s="8" t="s">
         <v>962</v>
       </c>
@@ -19675,7 +19716,7 @@
       <c r="B200" s="8">
         <v>4</v>
       </c>
-      <c r="C200" s="53"/>
+      <c r="C200" s="41"/>
       <c r="D200" s="8" t="s">
         <v>937</v>
       </c>
@@ -19687,13 +19728,13 @@
       <c r="B201" s="8">
         <v>11</v>
       </c>
-      <c r="C201" s="53" t="s">
+      <c r="C201" s="41" t="s">
         <v>1219</v>
       </c>
       <c r="D201" s="8" t="s">
         <v>931</v>
       </c>
-      <c r="E201" s="53"/>
+      <c r="E201" s="41"/>
     </row>
     <row r="202" spans="1:5">
       <c r="A202" s="8" t="s">
@@ -19702,7 +19743,7 @@
       <c r="B202" s="8">
         <v>1</v>
       </c>
-      <c r="C202" s="53"/>
+      <c r="C202" s="41"/>
       <c r="D202" s="8" t="s">
         <v>931</v>
       </c>
@@ -19714,7 +19755,7 @@
       <c r="B203" s="8">
         <v>3</v>
       </c>
-      <c r="C203" s="53" t="s">
+      <c r="C203" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D203" s="8" t="s">
@@ -19728,7 +19769,7 @@
       <c r="B204" s="8">
         <v>9</v>
       </c>
-      <c r="C204" s="53"/>
+      <c r="C204" s="41"/>
       <c r="D204" s="8" t="s">
         <v>931</v>
       </c>
@@ -19740,7 +19781,7 @@
       <c r="B205" s="8">
         <v>2</v>
       </c>
-      <c r="C205" s="53"/>
+      <c r="C205" s="41"/>
       <c r="D205" s="8" t="s">
         <v>931</v>
       </c>
@@ -19752,7 +19793,7 @@
       <c r="B206" s="8">
         <v>37</v>
       </c>
-      <c r="C206" s="53"/>
+      <c r="C206" s="41"/>
       <c r="D206" s="8" t="s">
         <v>931</v>
       </c>
@@ -19764,7 +19805,7 @@
       <c r="B207" s="8">
         <v>1</v>
       </c>
-      <c r="C207" s="53"/>
+      <c r="C207" s="41"/>
       <c r="D207" s="8" t="s">
         <v>931</v>
       </c>
@@ -19776,7 +19817,7 @@
       <c r="B208" s="8">
         <v>1</v>
       </c>
-      <c r="C208" s="53" t="s">
+      <c r="C208" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D208" s="8" t="s">
@@ -19790,7 +19831,7 @@
       <c r="B209" s="8">
         <v>1</v>
       </c>
-      <c r="C209" s="53" t="s">
+      <c r="C209" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D209" s="8" t="s">
@@ -19804,7 +19845,7 @@
       <c r="B210" s="8">
         <v>9</v>
       </c>
-      <c r="C210" s="53"/>
+      <c r="C210" s="41"/>
       <c r="D210" s="8" t="s">
         <v>931</v>
       </c>
@@ -19816,7 +19857,7 @@
       <c r="B211" s="8">
         <v>2</v>
       </c>
-      <c r="C211" s="53" t="s">
+      <c r="C211" s="41" t="s">
         <v>957</v>
       </c>
       <c r="D211" s="8" t="s">
@@ -19830,7 +19871,7 @@
       <c r="B212" s="8">
         <v>7</v>
       </c>
-      <c r="C212" s="53"/>
+      <c r="C212" s="41"/>
       <c r="D212" s="8" t="s">
         <v>931</v>
       </c>
@@ -19842,7 +19883,7 @@
       <c r="B213" s="8">
         <v>10</v>
       </c>
-      <c r="C213" s="53"/>
+      <c r="C213" s="41"/>
       <c r="D213" s="8" t="s">
         <v>965</v>
       </c>
@@ -19854,7 +19895,7 @@
       <c r="B214" s="8">
         <v>1</v>
       </c>
-      <c r="C214" s="53"/>
+      <c r="C214" s="41"/>
       <c r="D214" s="8" t="s">
         <v>934</v>
       </c>
@@ -19866,7 +19907,7 @@
       <c r="B215" s="8">
         <v>2</v>
       </c>
-      <c r="C215" s="53"/>
+      <c r="C215" s="41"/>
       <c r="D215" s="8" t="s">
         <v>931</v>
       </c>
@@ -19878,7 +19919,7 @@
       <c r="B216" s="8">
         <v>4</v>
       </c>
-      <c r="C216" s="53" t="s">
+      <c r="C216" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D216" s="8" t="s">
@@ -19892,7 +19933,7 @@
       <c r="B217" s="8">
         <v>5</v>
       </c>
-      <c r="C217" s="53" t="s">
+      <c r="C217" s="41" t="s">
         <v>970</v>
       </c>
       <c r="D217" s="8" t="s">
@@ -19906,7 +19947,7 @@
       <c r="B218" s="8">
         <v>17</v>
       </c>
-      <c r="C218" s="53" t="s">
+      <c r="C218" s="41" t="s">
         <v>972</v>
       </c>
       <c r="D218" s="8" t="s">
@@ -19920,7 +19961,7 @@
       <c r="B219" s="8">
         <v>1</v>
       </c>
-      <c r="C219" s="53"/>
+      <c r="C219" s="41"/>
       <c r="D219" s="8" t="s">
         <v>937</v>
       </c>
@@ -19932,7 +19973,7 @@
       <c r="B220" s="8">
         <v>1</v>
       </c>
-      <c r="C220" s="53"/>
+      <c r="C220" s="41"/>
       <c r="D220" s="8" t="s">
         <v>931</v>
       </c>
@@ -19944,7 +19985,7 @@
       <c r="B221" s="8">
         <v>1</v>
       </c>
-      <c r="C221" s="53" t="s">
+      <c r="C221" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D221" s="8" t="s">
@@ -19958,7 +19999,7 @@
       <c r="B222" s="8">
         <v>1</v>
       </c>
-      <c r="C222" s="53"/>
+      <c r="C222" s="41"/>
       <c r="D222" s="8" t="s">
         <v>931</v>
       </c>
@@ -19970,7 +20011,7 @@
       <c r="B223" s="8">
         <v>1</v>
       </c>
-      <c r="C223" s="53"/>
+      <c r="C223" s="41"/>
       <c r="D223" s="8" t="s">
         <v>931</v>
       </c>
@@ -19982,7 +20023,7 @@
       <c r="B224" s="8">
         <v>17</v>
       </c>
-      <c r="C224" s="53" t="s">
+      <c r="C224" s="41" t="s">
         <v>979</v>
       </c>
       <c r="D224" s="8" t="s">
@@ -19996,7 +20037,7 @@
       <c r="B225" s="8">
         <v>3</v>
       </c>
-      <c r="C225" s="53"/>
+      <c r="C225" s="41"/>
       <c r="D225" s="8" t="s">
         <v>934</v>
       </c>
@@ -20008,7 +20049,7 @@
       <c r="B226" s="8">
         <v>1</v>
       </c>
-      <c r="C226" s="53"/>
+      <c r="C226" s="41"/>
       <c r="D226" s="8" t="s">
         <v>740</v>
       </c>
@@ -20020,7 +20061,7 @@
       <c r="B227" s="8">
         <v>2</v>
       </c>
-      <c r="C227" s="53"/>
+      <c r="C227" s="41"/>
       <c r="D227" s="8" t="s">
         <v>740</v>
       </c>
@@ -20032,7 +20073,7 @@
       <c r="B228" s="8" t="s">
         <v>995</v>
       </c>
-      <c r="C228" s="53" t="s">
+      <c r="C228" s="41" t="s">
         <v>994</v>
       </c>
       <c r="D228" s="8" t="s">
@@ -20046,7 +20087,7 @@
       <c r="B229" s="8">
         <v>1</v>
       </c>
-      <c r="C229" s="53"/>
+      <c r="C229" s="41"/>
       <c r="D229" s="8" t="s">
         <v>931</v>
       </c>
@@ -20058,7 +20099,7 @@
       <c r="B230" s="8">
         <v>9</v>
       </c>
-      <c r="C230" s="53"/>
+      <c r="C230" s="41"/>
       <c r="D230" s="8" t="s">
         <v>931</v>
       </c>
@@ -20070,7 +20111,7 @@
       <c r="B231" s="8">
         <v>1</v>
       </c>
-      <c r="C231" s="53"/>
+      <c r="C231" s="41"/>
       <c r="D231" s="8" t="s">
         <v>934</v>
       </c>
@@ -20082,7 +20123,7 @@
       <c r="B232" s="8">
         <v>1</v>
       </c>
-      <c r="C232" s="53" t="s">
+      <c r="C232" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D232" s="8" t="s">
@@ -20096,7 +20137,7 @@
       <c r="B233" s="8">
         <v>2</v>
       </c>
-      <c r="C233" s="53"/>
+      <c r="C233" s="41"/>
       <c r="D233" s="8" t="s">
         <v>931</v>
       </c>
@@ -20108,7 +20149,7 @@
       <c r="B234" s="8">
         <v>11</v>
       </c>
-      <c r="C234" s="53"/>
+      <c r="C234" s="41"/>
       <c r="D234" s="8" t="s">
         <v>740</v>
       </c>
@@ -20120,7 +20161,7 @@
       <c r="B235" s="8">
         <v>1</v>
       </c>
-      <c r="C235" s="53"/>
+      <c r="C235" s="41"/>
       <c r="D235" s="8" t="s">
         <v>931</v>
       </c>
@@ -20132,7 +20173,7 @@
       <c r="B236" s="8">
         <v>10</v>
       </c>
-      <c r="C236" s="53" t="s">
+      <c r="C236" s="41" t="s">
         <v>991</v>
       </c>
       <c r="D236" s="8" t="s">
@@ -20146,7 +20187,7 @@
       <c r="B237" s="8">
         <v>7</v>
       </c>
-      <c r="C237" s="53"/>
+      <c r="C237" s="41"/>
       <c r="D237" s="8" t="s">
         <v>934</v>
       </c>
@@ -20158,7 +20199,7 @@
       <c r="B238" s="8">
         <v>4</v>
       </c>
-      <c r="C238" s="53"/>
+      <c r="C238" s="41"/>
       <c r="D238" s="8" t="s">
         <v>937</v>
       </c>
@@ -20170,7 +20211,7 @@
       <c r="B239" s="8">
         <v>1</v>
       </c>
-      <c r="C239" s="53"/>
+      <c r="C239" s="41"/>
       <c r="D239" s="8" t="s">
         <v>931</v>
       </c>
@@ -20182,7 +20223,7 @@
       <c r="B240" s="8">
         <v>16</v>
       </c>
-      <c r="C240" s="53"/>
+      <c r="C240" s="41"/>
       <c r="D240" s="8" t="s">
         <v>934</v>
       </c>
@@ -20194,7 +20235,7 @@
       <c r="B241" s="8">
         <v>15</v>
       </c>
-      <c r="C241" s="53"/>
+      <c r="C241" s="41"/>
       <c r="D241" s="8" t="s">
         <v>931</v>
       </c>
@@ -20206,7 +20247,7 @@
       <c r="B242" s="8">
         <v>2</v>
       </c>
-      <c r="C242" s="53"/>
+      <c r="C242" s="41"/>
       <c r="D242" s="8" t="s">
         <v>931</v>
       </c>
@@ -20218,7 +20259,7 @@
       <c r="B243" s="8">
         <v>53</v>
       </c>
-      <c r="C243" s="53" t="s">
+      <c r="C243" s="41" t="s">
         <v>1002</v>
       </c>
       <c r="D243" s="8" t="s">
@@ -20232,7 +20273,7 @@
       <c r="B244" s="8">
         <v>1</v>
       </c>
-      <c r="C244" s="53"/>
+      <c r="C244" s="41"/>
       <c r="D244" s="8" t="s">
         <v>740</v>
       </c>
@@ -20244,7 +20285,7 @@
       <c r="B245" s="8">
         <v>2</v>
       </c>
-      <c r="C245" s="53"/>
+      <c r="C245" s="41"/>
       <c r="D245" s="8" t="s">
         <v>934</v>
       </c>
@@ -20256,7 +20297,7 @@
       <c r="B246" s="8">
         <v>1</v>
       </c>
-      <c r="C246" s="53"/>
+      <c r="C246" s="41"/>
       <c r="D246" s="8" t="s">
         <v>931</v>
       </c>
@@ -20268,7 +20309,7 @@
       <c r="B247" s="8">
         <v>20</v>
       </c>
-      <c r="C247" s="53" t="s">
+      <c r="C247" s="41" t="s">
         <v>1021</v>
       </c>
       <c r="D247" s="8" t="s">
@@ -20282,7 +20323,7 @@
       <c r="B248" s="8">
         <v>6</v>
       </c>
-      <c r="C248" s="53" t="s">
+      <c r="C248" s="41" t="s">
         <v>1220</v>
       </c>
       <c r="D248" s="8" t="s">
@@ -20296,7 +20337,7 @@
       <c r="B249" s="8">
         <v>2</v>
       </c>
-      <c r="C249" s="53" t="s">
+      <c r="C249" s="41" t="s">
         <v>957</v>
       </c>
       <c r="D249" s="8" t="s">
@@ -20310,7 +20351,7 @@
       <c r="B250" s="8">
         <v>1</v>
       </c>
-      <c r="C250" s="53"/>
+      <c r="C250" s="41"/>
       <c r="D250" s="8" t="s">
         <v>934</v>
       </c>
@@ -20322,7 +20363,7 @@
       <c r="B251" s="8">
         <v>1</v>
       </c>
-      <c r="C251" s="53"/>
+      <c r="C251" s="41"/>
       <c r="D251" s="8" t="s">
         <v>931</v>
       </c>
@@ -20334,7 +20375,7 @@
       <c r="B252" s="8">
         <v>6</v>
       </c>
-      <c r="C252" s="53"/>
+      <c r="C252" s="41"/>
       <c r="D252" s="8" t="s">
         <v>934</v>
       </c>
@@ -20346,7 +20387,7 @@
       <c r="B253" s="8">
         <v>1</v>
       </c>
-      <c r="C253" s="53"/>
+      <c r="C253" s="41"/>
       <c r="D253" s="8" t="s">
         <v>934</v>
       </c>
@@ -20358,7 +20399,7 @@
       <c r="B254" s="8">
         <v>1</v>
       </c>
-      <c r="C254" s="53"/>
+      <c r="C254" s="41"/>
       <c r="D254" s="8" t="s">
         <v>931</v>
       </c>
@@ -20370,7 +20411,7 @@
       <c r="B255" s="8">
         <v>26</v>
       </c>
-      <c r="C255" s="53"/>
+      <c r="C255" s="41"/>
       <c r="D255" s="8" t="s">
         <v>937</v>
       </c>
@@ -20382,7 +20423,7 @@
       <c r="B256" s="8">
         <v>46</v>
       </c>
-      <c r="C256" s="53" t="s">
+      <c r="C256" s="41" t="s">
         <v>1016</v>
       </c>
       <c r="D256" s="8" t="s">
@@ -20396,7 +20437,7 @@
       <c r="B257" s="8">
         <v>10</v>
       </c>
-      <c r="C257" s="53" t="s">
+      <c r="C257" s="41" t="s">
         <v>991</v>
       </c>
       <c r="D257" s="8" t="s">
@@ -20410,7 +20451,7 @@
       <c r="B258" s="8">
         <v>6</v>
       </c>
-      <c r="C258" s="53"/>
+      <c r="C258" s="41"/>
       <c r="D258" s="8" t="s">
         <v>740</v>
       </c>
@@ -20422,7 +20463,7 @@
       <c r="B259" s="8">
         <v>1</v>
       </c>
-      <c r="C259" s="53"/>
+      <c r="C259" s="41"/>
       <c r="D259" s="8" t="s">
         <v>740</v>
       </c>
@@ -20434,7 +20475,7 @@
       <c r="B260" s="8">
         <v>4</v>
       </c>
-      <c r="C260" s="53"/>
+      <c r="C260" s="41"/>
       <c r="D260" s="8" t="s">
         <v>934</v>
       </c>
@@ -20446,7 +20487,7 @@
       <c r="B261" s="8">
         <v>2</v>
       </c>
-      <c r="C261" s="53" t="s">
+      <c r="C261" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D261" s="8" t="s">
@@ -20460,7 +20501,7 @@
       <c r="B262" s="8">
         <v>1</v>
       </c>
-      <c r="C262" s="53" t="s">
+      <c r="C262" s="41" t="s">
         <v>1024</v>
       </c>
       <c r="D262" s="8" t="s">
@@ -20474,7 +20515,7 @@
       <c r="B263" s="8">
         <v>3</v>
       </c>
-      <c r="C263" s="53" t="s">
+      <c r="C263" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D263" s="8" t="s">
@@ -20488,7 +20529,7 @@
       <c r="B264" s="8">
         <v>1</v>
       </c>
-      <c r="C264" s="53" t="s">
+      <c r="C264" s="41" t="s">
         <v>948</v>
       </c>
       <c r="D264" s="8" t="s">
@@ -20502,7 +20543,7 @@
       <c r="B265" s="8">
         <v>5</v>
       </c>
-      <c r="C265" s="53" t="s">
+      <c r="C265" s="41" t="s">
         <v>1028</v>
       </c>
       <c r="D265" s="8" t="s">
@@ -20516,19 +20557,19 @@
       <c r="B266" s="8">
         <v>8</v>
       </c>
-      <c r="C266" s="53"/>
+      <c r="C266" s="41"/>
       <c r="D266" s="8" t="s">
         <v>931</v>
       </c>
     </row>
     <row r="267" spans="1:5" ht="31">
-      <c r="A267" s="54" t="s">
+      <c r="A267" s="42" t="s">
         <v>256</v>
       </c>
       <c r="B267" s="8"/>
-      <c r="C267" s="53"/>
+      <c r="C267" s="41"/>
       <c r="D267" s="8"/>
-      <c r="E267" s="53" t="s">
+      <c r="E267" s="41" t="s">
         <v>963</v>
       </c>
     </row>
@@ -20539,7 +20580,7 @@
       <c r="B268" s="8">
         <v>4</v>
       </c>
-      <c r="C268" s="53"/>
+      <c r="C268" s="41"/>
       <c r="D268" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20551,7 +20592,7 @@
       <c r="B269" s="8">
         <v>1</v>
       </c>
-      <c r="C269" s="53" t="s">
+      <c r="C269" s="41" t="s">
         <v>1032</v>
       </c>
       <c r="D269" s="8" t="s">
@@ -20565,7 +20606,7 @@
       <c r="B270" s="8">
         <v>1</v>
       </c>
-      <c r="C270" s="53" t="s">
+      <c r="C270" s="41" t="s">
         <v>1035</v>
       </c>
       <c r="D270" s="8" t="s">
@@ -20579,7 +20620,7 @@
       <c r="B271" s="8">
         <v>6</v>
       </c>
-      <c r="C271" s="53"/>
+      <c r="C271" s="41"/>
       <c r="D271" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20591,7 +20632,7 @@
       <c r="B272" s="8">
         <v>69</v>
       </c>
-      <c r="C272" s="53" t="s">
+      <c r="C272" s="41" t="s">
         <v>1038</v>
       </c>
       <c r="D272" s="8" t="s">
@@ -20605,7 +20646,7 @@
       <c r="B273" s="8">
         <v>1</v>
       </c>
-      <c r="C273" s="53"/>
+      <c r="C273" s="41"/>
       <c r="D273" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20617,7 +20658,7 @@
       <c r="B274" s="8" t="s">
         <v>1041</v>
       </c>
-      <c r="C274" s="53" t="s">
+      <c r="C274" s="41" t="s">
         <v>1042</v>
       </c>
       <c r="D274" s="8" t="s">
@@ -20627,7 +20668,7 @@
     <row r="275" spans="1:5">
       <c r="A275" s="8"/>
       <c r="B275" s="8"/>
-      <c r="C275" s="53" t="s">
+      <c r="C275" s="41" t="s">
         <v>1002</v>
       </c>
       <c r="D275" s="8" t="s">
@@ -20641,7 +20682,7 @@
       <c r="B276" s="8" t="s">
         <v>1046</v>
       </c>
-      <c r="C276" s="53" t="s">
+      <c r="C276" s="41" t="s">
         <v>1090</v>
       </c>
       <c r="D276" s="8" t="s">
@@ -20655,7 +20696,7 @@
       <c r="B277" s="8" t="s">
         <v>1048</v>
       </c>
-      <c r="C277" s="53"/>
+      <c r="C277" s="41"/>
       <c r="D277" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20667,7 +20708,7 @@
       <c r="B278" s="8">
         <v>29</v>
       </c>
-      <c r="C278" s="53"/>
+      <c r="C278" s="41"/>
       <c r="D278" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20679,7 +20720,7 @@
       <c r="B279" s="8">
         <v>1</v>
       </c>
-      <c r="C279" s="53"/>
+      <c r="C279" s="41"/>
       <c r="D279" s="8" t="s">
         <v>1033</v>
       </c>
@@ -20688,7 +20729,7 @@
       <c r="A280" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="E280" s="53" t="s">
+      <c r="E280" s="41" t="s">
         <v>1197</v>
       </c>
     </row>
@@ -20699,7 +20740,7 @@
       <c r="B281" s="8">
         <v>1</v>
       </c>
-      <c r="C281" s="53"/>
+      <c r="C281" s="41"/>
       <c r="D281" s="8" t="s">
         <v>1051</v>
       </c>
@@ -20717,7 +20758,7 @@
       <c r="D282" t="s">
         <v>1051</v>
       </c>
-      <c r="E282" s="53" t="s">
+      <c r="E282" s="41" t="s">
         <v>556</v>
       </c>
     </row>
@@ -20773,7 +20814,7 @@
       <c r="B286" s="8">
         <v>9</v>
       </c>
-      <c r="C286" s="53"/>
+      <c r="C286" s="41"/>
       <c r="D286" s="8" t="s">
         <v>1055</v>
       </c>
@@ -20802,7 +20843,7 @@
       <c r="B288" s="8">
         <v>4</v>
       </c>
-      <c r="C288" s="53"/>
+      <c r="C288" s="41"/>
       <c r="D288" s="8" t="s">
         <v>740</v>
       </c>
@@ -20814,7 +20855,7 @@
       <c r="B289" s="8">
         <v>2</v>
       </c>
-      <c r="C289" s="53"/>
+      <c r="C289" s="41"/>
       <c r="D289" s="8" t="s">
         <v>1055</v>
       </c>
@@ -20840,7 +20881,7 @@
       <c r="B291" s="8">
         <v>47</v>
       </c>
-      <c r="C291" s="53" t="s">
+      <c r="C291" s="41" t="s">
         <v>1057</v>
       </c>
       <c r="D291" s="8" t="s">
@@ -20857,7 +20898,7 @@
       <c r="B292" s="8">
         <v>1</v>
       </c>
-      <c r="C292" s="53"/>
+      <c r="C292" s="41"/>
       <c r="D292" s="8" t="s">
         <v>740</v>
       </c>
@@ -20869,7 +20910,7 @@
       <c r="B293" s="8">
         <v>1</v>
       </c>
-      <c r="C293" s="53"/>
+      <c r="C293" s="41"/>
       <c r="D293" s="8" t="s">
         <v>1058</v>
       </c>
@@ -20929,13 +20970,13 @@
       <c r="B297" s="8">
         <v>80</v>
       </c>
-      <c r="C297" s="53" t="s">
+      <c r="C297" s="41" t="s">
         <v>1094</v>
       </c>
       <c r="D297" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E297" s="53" t="s">
+      <c r="E297" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -20946,7 +20987,7 @@
       <c r="B298" s="8">
         <v>13</v>
       </c>
-      <c r="C298" s="53"/>
+      <c r="C298" s="41"/>
       <c r="D298" s="8" t="s">
         <v>1051</v>
       </c>
@@ -20994,7 +21035,7 @@
       <c r="B302" s="8">
         <v>52</v>
       </c>
-      <c r="C302" s="53" t="s">
+      <c r="C302" s="41" t="s">
         <v>739</v>
       </c>
       <c r="D302" s="8" t="s">
@@ -21056,11 +21097,11 @@
       <c r="B306" s="8">
         <v>8</v>
       </c>
-      <c r="C306" s="53"/>
+      <c r="C306" s="41"/>
       <c r="D306" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E306" s="53" t="s">
+      <c r="E306" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21071,11 +21112,11 @@
       <c r="B307" s="8">
         <v>1</v>
       </c>
-      <c r="C307" s="53"/>
+      <c r="C307" s="41"/>
       <c r="D307" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E307" s="53" t="s">
+      <c r="E307" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21086,11 +21127,11 @@
       <c r="B308" s="8">
         <v>11</v>
       </c>
-      <c r="C308" s="53"/>
+      <c r="C308" s="41"/>
       <c r="D308" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E308" s="53" t="s">
+      <c r="E308" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21101,11 +21142,11 @@
       <c r="B309" s="8">
         <v>1</v>
       </c>
-      <c r="C309" s="53"/>
+      <c r="C309" s="41"/>
       <c r="D309" s="8" t="s">
         <v>1088</v>
       </c>
-      <c r="E309" s="53" t="s">
+      <c r="E309" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21116,11 +21157,11 @@
       <c r="B310" s="8">
         <v>23</v>
       </c>
-      <c r="C310" s="53"/>
+      <c r="C310" s="41"/>
       <c r="D310" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E310" s="53" t="s">
+      <c r="E310" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21131,13 +21172,13 @@
       <c r="B311" s="8">
         <v>24</v>
       </c>
-      <c r="C311" s="53" t="s">
+      <c r="C311" s="41" t="s">
         <v>1061</v>
       </c>
       <c r="D311" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E311" s="53" t="s">
+      <c r="E311" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21148,11 +21189,11 @@
       <c r="B312" s="8">
         <v>6</v>
       </c>
-      <c r="C312" s="53"/>
+      <c r="C312" s="41"/>
       <c r="D312" s="8" t="s">
         <v>1051</v>
       </c>
-      <c r="E312" s="53" t="s">
+      <c r="E312" s="41" t="s">
         <v>1189</v>
       </c>
     </row>
@@ -21247,7 +21288,7 @@
       <c r="B319" s="8">
         <v>6</v>
       </c>
-      <c r="C319" s="53"/>
+      <c r="C319" s="41"/>
       <c r="D319" s="8" t="s">
         <v>1055</v>
       </c>
@@ -21279,7 +21320,7 @@
       <c r="B321" s="8">
         <v>50</v>
       </c>
-      <c r="C321" s="53"/>
+      <c r="C321" s="41"/>
       <c r="D321" s="8" t="s">
         <v>1051</v>
       </c>
@@ -21316,7 +21357,7 @@
       <c r="B324" s="8">
         <v>6</v>
       </c>
-      <c r="C324" s="53"/>
+      <c r="C324" s="41"/>
       <c r="D324" s="8" t="s">
         <v>1051</v>
       </c>
@@ -21434,7 +21475,7 @@
       <c r="B333" s="8">
         <v>13</v>
       </c>
-      <c r="C333" s="53" t="s">
+      <c r="C333" s="41" t="s">
         <v>1101</v>
       </c>
       <c r="D333" s="8" t="s">
@@ -21451,7 +21492,7 @@
       <c r="B334" s="8">
         <v>4</v>
       </c>
-      <c r="C334" s="53"/>
+      <c r="C334" s="41"/>
       <c r="D334" s="8" t="s">
         <v>740</v>
       </c>
@@ -21524,7 +21565,7 @@
       <c r="B340" s="8">
         <v>7</v>
       </c>
-      <c r="C340" s="53"/>
+      <c r="C340" s="41"/>
       <c r="D340" s="8" t="s">
         <v>1055</v>
       </c>
@@ -21578,7 +21619,7 @@
       <c r="B344" s="8">
         <v>111</v>
       </c>
-      <c r="C344" s="53" t="s">
+      <c r="C344" s="41" t="s">
         <v>1061</v>
       </c>
       <c r="D344" s="8" t="s">
@@ -21636,13 +21677,13 @@
       <c r="B349" s="8">
         <v>27</v>
       </c>
-      <c r="C349" s="53" t="s">
+      <c r="C349" s="41" t="s">
         <v>1221</v>
       </c>
       <c r="D349" s="8" t="s">
         <v>1144</v>
       </c>
-      <c r="E349" s="53" t="s">
+      <c r="E349" s="41" t="s">
         <v>1222</v>
       </c>
     </row>
@@ -21945,13 +21986,13 @@
       </c>
     </row>
     <row r="374" spans="1:5" ht="78" customHeight="1">
-      <c r="A374" s="65" t="s">
+      <c r="A374" s="53" t="s">
         <v>1260</v>
       </c>
-      <c r="B374" s="65"/>
-      <c r="C374" s="65"/>
-      <c r="D374" s="65"/>
-      <c r="E374" s="65"/>
+      <c r="B374" s="53"/>
+      <c r="C374" s="53"/>
+      <c r="D374" s="53"/>
+      <c r="E374" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -22010,7 +22051,7 @@
       <c r="A6" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="49" t="s">
         <v>1286</v>
       </c>
     </row>
@@ -22042,7 +22083,7 @@
       <c r="A10" s="26" t="s">
         <v>547</v>
       </c>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="49" t="s">
         <v>1285</v>
       </c>
     </row>
@@ -22095,23 +22136,23 @@
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="61"/>
+      <c r="A18" s="49"/>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="49" t="s">
         <v>1254</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="49" t="s">
         <v>1255</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="49" t="s">
         <v>1288</v>
       </c>
     </row>

</xml_diff>

<commit_message>
modified:   data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx 	new file:   data/chapter2/FRED/subsets/species.txt 	modified:   data/chapter2/FRED/subsets/species.xlsx 	deleted:    data/chapter2/FRED/subsets/states.txt 	new file:   data/chapter2/Wang & Qiu - 2006 - Table1.html 	new file:   notebooks/chapter_02/Wang & Qiu 2006.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
+++ b/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF889681-845B-4B0E-AD38-94737A5407DF}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56EA462F-12E2-488D-A9D7-FFA93E862D54}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Information" sheetId="7" r:id="rId1"/>
@@ -4720,12 +4720,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -4741,6 +4735,12 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -4748,12 +4748,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -4803,13 +4797,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFC4D79B"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color rgb="FFC4D79B"/>
         </left>
@@ -4820,6 +4807,19 @@
           <color rgb="FFC4D79B"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFC4D79B"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -4858,6 +4858,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I439" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A1:I439" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -4880,18 +4884,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2922BC0C-E417-4658-AC0E-62ECDF39ADC6}" name="Table2" displayName="Table2" ref="A2:F89" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="8" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2922BC0C-E417-4658-AC0E-62ECDF39ADC6}" name="Table2" displayName="Table2" ref="A2:F89" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6">
   <autoFilter ref="A2:F89" xr:uid="{2922BC0C-E417-4658-AC0E-62ECDF39ADC6}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F89">
     <sortCondition ref="B2:B89"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0BA76706-F6AC-4480-A1EA-EFC458A86717}" name="Order" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{5641DCB1-A433-40BD-9ED9-D33902929B8C}" name="Family" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{DAAE68C8-09E1-4B56-912D-11D87EB83220}" name="Habit" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{2BC3EF26-068C-475F-91C7-4E8D11F95517}" name="Ecology" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{C1FBDF6D-8E5A-4A09-BBA3-846E464D6CA5}" name="NM-AM" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{0B4BCA8E-55FF-4900-A159-74CFB7CBAE73}" name="NM" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{0BA76706-F6AC-4480-A1EA-EFC458A86717}" name="Order" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{5641DCB1-A433-40BD-9ED9-D33902929B8C}" name="Family" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{DAAE68C8-09E1-4B56-912D-11D87EB83220}" name="Habit" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{2BC3EF26-068C-475F-91C7-4E8D11F95517}" name="Ecology" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C1FBDF6D-8E5A-4A09-BBA3-846E464D6CA5}" name="NM-AM" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{0B4BCA8E-55FF-4900-A159-74CFB7CBAE73}" name="NM" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5329,7 +5333,7 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="18.5" customWidth="1"/>
-    <col min="2" max="2" width="24.5" customWidth="1"/>
+    <col min="2" max="2" width="32.4140625" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" customWidth="1"/>
@@ -15625,35 +15629,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="82" customHeight="1" thickBot="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="57" t="s">
         <v>560</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
       <c r="G1" s="8" t="s">
         <v>1261</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" thickBot="1">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="58" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="58" t="s">
+      <c r="B2" s="56" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="56" t="s">
         <v>561</v>
       </c>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="56" t="s">
         <v>562</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="58" t="s">
+      <c r="F2" s="56" t="s">
         <v>12</v>
       </c>
     </row>
@@ -15673,7 +15677,7 @@
       <c r="E3" s="36">
         <v>2</v>
       </c>
-      <c r="F3" s="55"/>
+      <c r="F3" s="53"/>
     </row>
     <row r="4" spans="1:7" ht="16" thickBot="1">
       <c r="A4" s="36" t="s">
@@ -15688,7 +15692,7 @@
       <c r="D4" s="36" t="s">
         <v>592</v>
       </c>
-      <c r="E4" s="55"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="36">
         <v>1900</v>
       </c>
@@ -15709,7 +15713,7 @@
       <c r="E5" s="35">
         <v>115</v>
       </c>
-      <c r="F5" s="54"/>
+      <c r="F5" s="52"/>
     </row>
     <row r="6" spans="1:7" ht="16" thickBot="1">
       <c r="A6" s="36" t="s">
@@ -15724,7 +15728,7 @@
       <c r="D6" s="36" t="s">
         <v>595</v>
       </c>
-      <c r="E6" s="55"/>
+      <c r="E6" s="53"/>
       <c r="F6" s="36">
         <v>2040</v>
       </c>
@@ -15742,7 +15746,7 @@
       <c r="D7" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E7" s="54"/>
+      <c r="E7" s="52"/>
       <c r="F7" s="35">
         <v>10</v>
       </c>
@@ -15763,7 +15767,7 @@
       <c r="E8" s="36">
         <v>56</v>
       </c>
-      <c r="F8" s="55"/>
+      <c r="F8" s="53"/>
     </row>
     <row r="9" spans="1:7" ht="16" thickBot="1">
       <c r="A9" s="35" t="s">
@@ -15781,7 +15785,7 @@
       <c r="E9" s="35">
         <v>1300</v>
       </c>
-      <c r="F9" s="54"/>
+      <c r="F9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="16" thickBot="1">
       <c r="A10" s="36" t="s">
@@ -15796,7 +15800,7 @@
       <c r="D10" s="36" t="s">
         <v>573</v>
       </c>
-      <c r="E10" s="55"/>
+      <c r="E10" s="53"/>
       <c r="F10" s="36">
         <v>8</v>
       </c>
@@ -15814,7 +15818,7 @@
       <c r="D11" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E11" s="54"/>
+      <c r="E11" s="52"/>
       <c r="F11" s="35">
         <v>39</v>
       </c>
@@ -15832,7 +15836,7 @@
       <c r="D12" s="35" t="s">
         <v>617</v>
       </c>
-      <c r="E12" s="54"/>
+      <c r="E12" s="52"/>
       <c r="F12" s="35">
         <v>3628</v>
       </c>
@@ -15850,10 +15854,10 @@
       <c r="D13" s="35" t="s">
         <v>570</v>
       </c>
-      <c r="E13" s="56">
+      <c r="E13" s="54">
         <v>3475</v>
       </c>
-      <c r="F13" s="54"/>
+      <c r="F13" s="52"/>
     </row>
     <row r="14" spans="1:7" ht="16" thickBot="1">
       <c r="A14" s="36" t="s">
@@ -15871,7 +15875,7 @@
       <c r="E14" s="36">
         <v>1</v>
       </c>
-      <c r="F14" s="55"/>
+      <c r="F14" s="53"/>
     </row>
     <row r="15" spans="1:7" ht="16" thickBot="1">
       <c r="A15" s="35" t="s">
@@ -15886,7 +15890,7 @@
       <c r="D15" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E15" s="54"/>
+      <c r="E15" s="52"/>
       <c r="F15" s="35">
         <v>8</v>
       </c>
@@ -15907,7 +15911,7 @@
       <c r="E16" s="36">
         <v>75</v>
       </c>
-      <c r="F16" s="55"/>
+      <c r="F16" s="53"/>
     </row>
     <row r="17" spans="1:6" ht="16" thickBot="1">
       <c r="A17" s="36" t="s">
@@ -15922,7 +15926,7 @@
       <c r="D17" s="36" t="s">
         <v>618</v>
       </c>
-      <c r="E17" s="55"/>
+      <c r="E17" s="53"/>
       <c r="F17" s="36">
         <v>450</v>
       </c>
@@ -15940,7 +15944,7 @@
       <c r="D18" s="35" t="s">
         <v>596</v>
       </c>
-      <c r="E18" s="54"/>
+      <c r="E18" s="52"/>
       <c r="F18" s="35">
         <v>2625</v>
       </c>
@@ -15958,7 +15962,7 @@
       <c r="D19" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E19" s="54"/>
+      <c r="E19" s="52"/>
       <c r="F19" s="35">
         <v>1</v>
       </c>
@@ -15976,7 +15980,7 @@
       <c r="D20" s="36" t="s">
         <v>564</v>
       </c>
-      <c r="E20" s="55"/>
+      <c r="E20" s="53"/>
       <c r="F20" s="36">
         <v>4</v>
       </c>
@@ -15994,7 +15998,7 @@
       <c r="D21" s="35" t="s">
         <v>592</v>
       </c>
-      <c r="E21" s="54"/>
+      <c r="E21" s="52"/>
       <c r="F21" s="35">
         <v>346</v>
       </c>
@@ -16012,7 +16016,7 @@
       <c r="D22" s="36" t="s">
         <v>577</v>
       </c>
-      <c r="E22" s="55"/>
+      <c r="E22" s="53"/>
       <c r="F22" s="36">
         <v>731</v>
       </c>
@@ -16030,7 +16034,7 @@
       <c r="D23" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E23" s="55"/>
+      <c r="E23" s="53"/>
       <c r="F23" s="36">
         <v>172</v>
       </c>
@@ -16071,7 +16075,7 @@
       <c r="E25" s="36">
         <v>230</v>
       </c>
-      <c r="F25" s="55"/>
+      <c r="F25" s="53"/>
     </row>
     <row r="26" spans="1:6" ht="16" thickBot="1">
       <c r="A26" s="35" t="s">
@@ -16086,7 +16090,7 @@
       <c r="D26" s="35" t="s">
         <v>573</v>
       </c>
-      <c r="E26" s="54"/>
+      <c r="E26" s="52"/>
       <c r="F26" s="35">
         <v>17</v>
       </c>
@@ -16104,7 +16108,7 @@
       <c r="D27" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E27" s="55"/>
+      <c r="E27" s="53"/>
       <c r="F27" s="36">
         <v>2</v>
       </c>
@@ -16125,7 +16129,7 @@
       <c r="E28" s="36">
         <v>5500</v>
       </c>
-      <c r="F28" s="55"/>
+      <c r="F28" s="53"/>
     </row>
     <row r="29" spans="1:6" ht="16" thickBot="1">
       <c r="A29" s="36" t="s">
@@ -16140,7 +16144,7 @@
       <c r="D29" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E29" s="55"/>
+      <c r="E29" s="53"/>
       <c r="F29" s="36">
         <v>10</v>
       </c>
@@ -16158,7 +16162,7 @@
       <c r="D30" s="35" t="s">
         <v>576</v>
       </c>
-      <c r="E30" s="54"/>
+      <c r="E30" s="52"/>
       <c r="F30" s="35">
         <v>16</v>
       </c>
@@ -16176,7 +16180,7 @@
       <c r="D31" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E31" s="54"/>
+      <c r="E31" s="52"/>
       <c r="F31" s="35">
         <v>180</v>
       </c>
@@ -16194,7 +16198,7 @@
       <c r="D32" s="36" t="s">
         <v>598</v>
       </c>
-      <c r="E32" s="55"/>
+      <c r="E32" s="53"/>
       <c r="F32" s="36">
         <v>1</v>
       </c>
@@ -16215,7 +16219,7 @@
       <c r="E33" s="36">
         <v>242</v>
       </c>
-      <c r="F33" s="55"/>
+      <c r="F33" s="53"/>
     </row>
     <row r="34" spans="1:6" ht="16" thickBot="1">
       <c r="A34" s="36" t="s">
@@ -16230,7 +16234,7 @@
       <c r="D34" s="36" t="s">
         <v>588</v>
       </c>
-      <c r="E34" s="55"/>
+      <c r="E34" s="53"/>
       <c r="F34" s="36">
         <v>700</v>
       </c>
@@ -16248,7 +16252,7 @@
       <c r="D35" s="35" t="s">
         <v>601</v>
       </c>
-      <c r="E35" s="54"/>
+      <c r="E35" s="52"/>
       <c r="F35" s="35">
         <v>90</v>
       </c>
@@ -16266,7 +16270,7 @@
       <c r="D36" s="35" t="s">
         <v>576</v>
       </c>
-      <c r="E36" s="54"/>
+      <c r="E36" s="52"/>
       <c r="F36" s="35">
         <v>102</v>
       </c>
@@ -16287,7 +16291,7 @@
       <c r="E37" s="36">
         <v>50</v>
       </c>
-      <c r="F37" s="55"/>
+      <c r="F37" s="53"/>
     </row>
     <row r="38" spans="1:6" ht="16" thickBot="1">
       <c r="A38" s="35" t="s">
@@ -16302,7 +16306,7 @@
       <c r="D38" s="35" t="s">
         <v>564</v>
       </c>
-      <c r="E38" s="54"/>
+      <c r="E38" s="52"/>
       <c r="F38" s="35">
         <v>3</v>
       </c>
@@ -16320,7 +16324,7 @@
       <c r="D39" s="35" t="s">
         <v>564</v>
       </c>
-      <c r="E39" s="54"/>
+      <c r="E39" s="52"/>
       <c r="F39" s="35">
         <v>12</v>
       </c>
@@ -16338,7 +16342,7 @@
       <c r="D40" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E40" s="55"/>
+      <c r="E40" s="53"/>
       <c r="F40" s="36">
         <v>7</v>
       </c>
@@ -16356,7 +16360,7 @@
       <c r="D41" s="36" t="s">
         <v>574</v>
       </c>
-      <c r="E41" s="55"/>
+      <c r="E41" s="53"/>
       <c r="F41" s="36">
         <v>135</v>
       </c>
@@ -16377,7 +16381,7 @@
       <c r="E42" s="35">
         <v>300</v>
       </c>
-      <c r="F42" s="54"/>
+      <c r="F42" s="52"/>
     </row>
     <row r="43" spans="1:6" ht="16" thickBot="1">
       <c r="A43" s="36" t="s">
@@ -16392,7 +16396,7 @@
       <c r="D43" s="36" t="s">
         <v>581</v>
       </c>
-      <c r="E43" s="55"/>
+      <c r="E43" s="53"/>
       <c r="F43" s="36">
         <v>464</v>
       </c>
@@ -16413,7 +16417,7 @@
       <c r="E44" s="35">
         <v>34</v>
       </c>
-      <c r="F44" s="54"/>
+      <c r="F44" s="52"/>
     </row>
     <row r="45" spans="1:6" ht="16" thickBot="1">
       <c r="A45" s="35" t="s">
@@ -16428,7 +16432,7 @@
       <c r="D45" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E45" s="54"/>
+      <c r="E45" s="52"/>
       <c r="F45" s="35">
         <v>19</v>
       </c>
@@ -16446,7 +16450,7 @@
       <c r="D46" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E46" s="55"/>
+      <c r="E46" s="53"/>
       <c r="F46" s="36">
         <v>4</v>
       </c>
@@ -16464,7 +16468,7 @@
       <c r="D47" s="36" t="s">
         <v>598</v>
       </c>
-      <c r="E47" s="55"/>
+      <c r="E47" s="53"/>
       <c r="F47" s="36">
         <v>316</v>
       </c>
@@ -16482,7 +16486,7 @@
       <c r="D48" s="36" t="s">
         <v>564</v>
       </c>
-      <c r="E48" s="55"/>
+      <c r="E48" s="53"/>
       <c r="F48" s="36">
         <v>8</v>
       </c>
@@ -16500,7 +16504,7 @@
       <c r="D49" s="36" t="s">
         <v>589</v>
       </c>
-      <c r="E49" s="55"/>
+      <c r="E49" s="53"/>
       <c r="F49" s="36">
         <v>308</v>
       </c>
@@ -16518,7 +16522,7 @@
       <c r="D50" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E50" s="54"/>
+      <c r="E50" s="52"/>
       <c r="F50" s="35">
         <v>1039</v>
       </c>
@@ -16539,7 +16543,7 @@
       <c r="E51" s="35">
         <v>60</v>
       </c>
-      <c r="F51" s="54"/>
+      <c r="F51" s="52"/>
     </row>
     <row r="52" spans="1:6" ht="16" thickBot="1">
       <c r="A52" s="36" t="s">
@@ -16554,7 +16558,7 @@
       <c r="D52" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E52" s="55"/>
+      <c r="E52" s="53"/>
       <c r="F52" s="36">
         <v>8</v>
       </c>
@@ -16572,7 +16576,7 @@
       <c r="D53" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E53" s="55"/>
+      <c r="E53" s="53"/>
       <c r="F53" s="36">
         <v>2</v>
       </c>
@@ -16590,7 +16594,7 @@
       <c r="D54" s="36" t="s">
         <v>602</v>
       </c>
-      <c r="E54" s="55"/>
+      <c r="E54" s="53"/>
       <c r="F54" s="36">
         <v>80</v>
       </c>
@@ -16608,7 +16612,7 @@
       <c r="D55" s="35" t="s">
         <v>585</v>
       </c>
-      <c r="E55" s="54"/>
+      <c r="E55" s="52"/>
       <c r="F55" s="35">
         <v>57</v>
       </c>
@@ -16626,7 +16630,7 @@
       <c r="D56" s="36" t="s">
         <v>564</v>
       </c>
-      <c r="E56" s="55"/>
+      <c r="E56" s="53"/>
       <c r="F56" s="36">
         <v>3</v>
       </c>
@@ -16644,7 +16648,7 @@
       <c r="D57" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E57" s="54"/>
+      <c r="E57" s="52"/>
       <c r="F57" s="35">
         <v>150</v>
       </c>
@@ -16662,7 +16666,7 @@
       <c r="D58" s="36" t="s">
         <v>227</v>
       </c>
-      <c r="E58" s="55"/>
+      <c r="E58" s="53"/>
       <c r="F58" s="36">
         <v>400</v>
       </c>
@@ -16683,7 +16687,7 @@
       <c r="E59" s="35">
         <v>70</v>
       </c>
-      <c r="F59" s="54"/>
+      <c r="F59" s="52"/>
     </row>
     <row r="60" spans="1:6" ht="16" thickBot="1">
       <c r="A60" s="36" t="s">
@@ -16698,7 +16702,7 @@
       <c r="D60" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E60" s="55"/>
+      <c r="E60" s="53"/>
       <c r="F60" s="36">
         <v>59</v>
       </c>
@@ -16716,7 +16720,7 @@
       <c r="D61" s="36" t="s">
         <v>567</v>
       </c>
-      <c r="E61" s="55"/>
+      <c r="E61" s="53"/>
       <c r="F61" s="36">
         <v>36</v>
       </c>
@@ -16734,7 +16738,7 @@
       <c r="D62" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E62" s="54"/>
+      <c r="E62" s="52"/>
       <c r="F62" s="35">
         <v>1957</v>
       </c>
@@ -16755,7 +16759,7 @@
       <c r="E63" s="35">
         <v>775</v>
       </c>
-      <c r="F63" s="54"/>
+      <c r="F63" s="52"/>
     </row>
     <row r="64" spans="1:6" ht="16" thickBot="1">
       <c r="A64" s="35" t="s">
@@ -16770,7 +16774,7 @@
       <c r="D64" s="35" t="s">
         <v>589</v>
       </c>
-      <c r="E64" s="54"/>
+      <c r="E64" s="52"/>
       <c r="F64" s="35">
         <v>33</v>
       </c>
@@ -16791,7 +16795,7 @@
       <c r="E65" s="35">
         <v>3700</v>
       </c>
-      <c r="F65" s="54"/>
+      <c r="F65" s="52"/>
     </row>
     <row r="66" spans="1:6" ht="16" thickBot="1">
       <c r="A66" s="36" t="s">
@@ -16809,7 +16813,7 @@
       <c r="E66" s="36">
         <v>725</v>
       </c>
-      <c r="F66" s="55"/>
+      <c r="F66" s="53"/>
     </row>
     <row r="67" spans="1:6" ht="16" thickBot="1">
       <c r="A67" s="35" t="s">
@@ -16827,7 +16831,7 @@
       <c r="E67" s="35">
         <v>300</v>
       </c>
-      <c r="F67" s="54"/>
+      <c r="F67" s="52"/>
     </row>
     <row r="68" spans="1:6" ht="16" thickBot="1">
       <c r="A68" s="35" t="s">
@@ -16842,7 +16846,7 @@
       <c r="D68" s="35" t="s">
         <v>589</v>
       </c>
-      <c r="E68" s="54"/>
+      <c r="E68" s="52"/>
       <c r="F68" s="35">
         <v>1200</v>
       </c>
@@ -16863,7 +16867,7 @@
       <c r="E69" s="36">
         <v>34</v>
       </c>
-      <c r="F69" s="55"/>
+      <c r="F69" s="53"/>
     </row>
     <row r="70" spans="1:6" ht="16" thickBot="1">
       <c r="A70" s="36" t="s">
@@ -16881,7 +16885,7 @@
       <c r="E70" s="36">
         <v>115</v>
       </c>
-      <c r="F70" s="55"/>
+      <c r="F70" s="53"/>
     </row>
     <row r="71" spans="1:6" ht="16" thickBot="1">
       <c r="A71" s="36" t="s">
@@ -16896,7 +16900,7 @@
       <c r="D71" s="36" t="s">
         <v>573</v>
       </c>
-      <c r="E71" s="55"/>
+      <c r="E71" s="53"/>
       <c r="F71" s="36">
         <v>9</v>
       </c>
@@ -16917,7 +16921,7 @@
       <c r="E72" s="35">
         <v>110</v>
       </c>
-      <c r="F72" s="54"/>
+      <c r="F72" s="52"/>
     </row>
     <row r="73" spans="1:6" ht="16" thickBot="1">
       <c r="A73" s="35" t="s">
@@ -16932,7 +16936,7 @@
       <c r="D73" s="35" t="s">
         <v>585</v>
       </c>
-      <c r="E73" s="54"/>
+      <c r="E73" s="52"/>
       <c r="F73" s="35">
         <v>1660</v>
       </c>
@@ -16950,7 +16954,7 @@
       <c r="D74" s="36" t="s">
         <v>227</v>
       </c>
-      <c r="E74" s="55"/>
+      <c r="E74" s="53"/>
       <c r="F74" s="36">
         <v>50</v>
       </c>
@@ -16968,7 +16972,7 @@
       <c r="D75" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E75" s="54"/>
+      <c r="E75" s="52"/>
       <c r="F75" s="35">
         <v>25</v>
       </c>
@@ -16986,7 +16990,7 @@
       <c r="D76" s="35" t="s">
         <v>619</v>
       </c>
-      <c r="E76" s="54"/>
+      <c r="E76" s="52"/>
       <c r="F76" s="35">
         <v>107</v>
       </c>
@@ -17004,7 +17008,7 @@
       <c r="D77" s="35" t="s">
         <v>583</v>
       </c>
-      <c r="E77" s="54"/>
+      <c r="E77" s="52"/>
       <c r="F77" s="35">
         <v>572</v>
       </c>
@@ -17025,7 +17029,7 @@
       <c r="E78" s="36">
         <v>147</v>
       </c>
-      <c r="F78" s="55"/>
+      <c r="F78" s="53"/>
     </row>
     <row r="79" spans="1:6" ht="16" thickBot="1">
       <c r="A79" s="35" t="s">
@@ -17040,8 +17044,8 @@
       <c r="D79" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E79" s="54"/>
-      <c r="F79" s="54"/>
+      <c r="E79" s="52"/>
+      <c r="F79" s="52"/>
     </row>
     <row r="80" spans="1:6" ht="16" thickBot="1">
       <c r="A80" s="36" t="s">
@@ -17056,7 +17060,7 @@
       <c r="D80" s="36" t="s">
         <v>574</v>
       </c>
-      <c r="E80" s="55"/>
+      <c r="E80" s="53"/>
       <c r="F80" s="36">
         <v>8</v>
       </c>
@@ -17074,7 +17078,7 @@
       <c r="D81" s="35" t="s">
         <v>567</v>
       </c>
-      <c r="E81" s="54"/>
+      <c r="E81" s="52"/>
       <c r="F81" s="35">
         <v>1097</v>
       </c>
@@ -17092,7 +17096,7 @@
       <c r="D82" s="35" t="s">
         <v>598</v>
       </c>
-      <c r="E82" s="54"/>
+      <c r="E82" s="52"/>
       <c r="F82" s="35">
         <v>34</v>
       </c>
@@ -17113,7 +17117,7 @@
       <c r="E83" s="35">
         <v>640</v>
       </c>
-      <c r="F83" s="54"/>
+      <c r="F83" s="52"/>
     </row>
     <row r="84" spans="1:6" ht="16" thickBot="1">
       <c r="A84" s="35" t="s">
@@ -17131,7 +17135,7 @@
       <c r="E84" s="35">
         <v>78</v>
       </c>
-      <c r="F84" s="54"/>
+      <c r="F84" s="52"/>
     </row>
     <row r="85" spans="1:6" ht="16" thickBot="1">
       <c r="A85" s="36" t="s">
@@ -17146,7 +17150,7 @@
       <c r="D85" s="36" t="s">
         <v>564</v>
       </c>
-      <c r="E85" s="55"/>
+      <c r="E85" s="53"/>
       <c r="F85" s="36">
         <v>51</v>
       </c>
@@ -17167,7 +17171,7 @@
       <c r="E86" s="36">
         <v>2625</v>
       </c>
-      <c r="F86" s="55"/>
+      <c r="F86" s="53"/>
     </row>
     <row r="87" spans="1:6" ht="16" thickBot="1">
       <c r="A87" s="35" t="s">
@@ -17182,7 +17186,7 @@
       <c r="D87" s="35" t="s">
         <v>564</v>
       </c>
-      <c r="E87" s="54"/>
+      <c r="E87" s="52"/>
       <c r="F87" s="35">
         <v>399</v>
       </c>
@@ -17200,7 +17204,7 @@
       <c r="D88" s="35" t="s">
         <v>573</v>
       </c>
-      <c r="E88" s="54"/>
+      <c r="E88" s="52"/>
       <c r="F88" s="35">
         <v>22</v>
       </c>
@@ -17221,7 +17225,7 @@
       <c r="E89" s="34">
         <v>285</v>
       </c>
-      <c r="F89" s="57"/>
+      <c r="F89" s="55"/>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="37" t="s">
@@ -21986,13 +21990,13 @@
       </c>
     </row>
     <row r="374" spans="1:5" ht="78" customHeight="1">
-      <c r="A374" s="53" t="s">
+      <c r="A374" s="58" t="s">
         <v>1260</v>
       </c>
-      <c r="B374" s="53"/>
-      <c r="C374" s="53"/>
-      <c r="D374" s="53"/>
-      <c r="E374" s="53"/>
+      <c r="B374" s="58"/>
+      <c r="C374" s="58"/>
+      <c r="D374" s="58"/>
+      <c r="E374" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
modified:   R/notebooks/MRPMM.ipynb 	modified:   data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx 	renamed:    data/chapter2/FRED/subsets/species.txt -> data/chapter2/FRED/subsets/species.changelog 	modified:   data/chapter2/FRED/subsets/species.xlsx
</commit_message>
<xml_diff>
--- a/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
+++ b/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56EA462F-12E2-488D-A9D7-FFA93E862D54}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9142FCD1-841D-46F7-BE01-F1D7C18E1826}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Information" sheetId="7" r:id="rId1"/>

</xml_diff>

<commit_message>
modified:   data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx 	modified:   data/chapter2/FRED/subsets/species.xlsx
</commit_message>
<xml_diff>
--- a/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
+++ b/data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9142FCD1-841D-46F7-BE01-F1D7C18E1826}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_9EE980E2FD5D26AFDFEDEA635E1132CB8726D636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{400E431F-0B84-4B76-8C78-E306B40FBEF0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Information" sheetId="7" r:id="rId1"/>

</xml_diff>